<commit_message>
Add completeness audit, process fixes, and diverse AI-idea column
- Completeness audit (20 critics): swap 10 weak/duplicate businesses for
  more recognizable, shareable ones; category balance preserved 1:1
- Review all 300 key-process descriptions; improve 50 (missing key step,
  bottleneck, or a factual contradiction)
- Add "Идея внедрения ИИ" column: one concrete idea per business tied to
  its bottleneck, diversified across a 28-type taxonomy (all 28 used, max
  27/300, chatbots only 2x), adversarially verified (16 corrections),
  0 duplicate ideas
- CSV now 8 columns (UTF-8 BOM) + XLSX; REVIEW note updated

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCSVxoQTm12nC9dfcVCB3G
</commit_message>
<xml_diff>
--- a/300_business_ai_cases.xlsx
+++ b/300_business_ai_cases.xlsx
@@ -435,16 +435,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G301"/>
+  <dimension ref="A1:H301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="66" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,6 +484,11 @@
           <t>Хук</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Идея внедрения ИИ</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -518,6 +524,11 @@
           <t>ИИ-консалтинг: где теряется прибыль, когда хайп продаётся быстрее, чем повторяемый и измеримый результат?</t>
         </is>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>ИИ-консалтинг: RAG-ассистент на базе прошлых проектов и регламентов подсказывает методику диагностики и типовые решения, стандартизирует результат и держит маржу без ручного контроля каждого консультанта.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -545,12 +556,17 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Изучаем спрос, закупаем партию, оформляем карточки товара, поставляем на склад площадки, продвигаем рекламой, отрабатываем возвраты и держим остатки под контролем.</t>
+          <t>Изучаем спрос и юнит-экономику, закупаем партию, оформляем карточки, поставляем на склад площадки, продвигаем рекламой и держим цену, отрабатываем возвраты и контролируем остатки.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Универсальный продавец на маркетплейсах: почему обороты растут, а денег на счёте всё меньше, если комиссия, логистика и невыкупленные заказы забирают половину наценки?</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Универсальный продавец на маркетплейсах: ИИ управляет ставками и бюджетами продвижения по каждой карточке на данных о выкупе и марже, снижает ДРР и возвращает наценку, съеденную рекламой.</t>
         </is>
       </c>
     </row>
@@ -588,6 +604,11 @@
           <t>SMM-агентство: что скрывается за красивым отчётом об охватах, если клиент не видит заявок и через пару месяцев молча уходит к конкурентам?</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>SMM-агентство: генеративный ИИ на бренд-гайдах клиента готовит черновики текстов и макетов контент-плана, снижает ручные часы команды на аккаунт и поднимает маржу абонентки.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -615,12 +636,17 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Ведём первичный приём, делаем снимок, составляем план лечения, записываем на этапы, лечим, ставим работу на гарантию и приглашаем на профосмотр.</t>
+          <t>Ведём первичный приём, делаем снимок, составляем план лечения и смету, согласуем стоимость, записываем на этапы, лечим, ставим работу на гарантию и зовём на профосмотр.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Стоматологическая клиника: куда утекает выручка, когда врач простаивает в пустом окне, пациент не пришёл на второй этап, а согласованный план остался на бумаге?</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Стоматологическая клиника: ИИ заполняет окна в расписании и достраивает загрузку кресел из очереди на несделанные этапы плана лечения, поднимает утилизацию кресел и сокращает простой врача.</t>
         </is>
       </c>
     </row>
@@ -658,6 +684,11 @@
           <t>Компания по ремонту квартир: сколько прибыли съедают переделки, простои бригад и внеплановая докупка материалов, если объект сдан в срок, а вышли почти в ноль?</t>
         </is>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Компания по ремонту квартир: ИИ собирает смету по замеру и истории объектов с актуальными ценами материалов, снижает плывущие сметы, переделки и внеплановую докупку, удерживая маржу объекта.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -685,12 +716,17 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Собираем требования, оцениваем трудозатраты, разбиваем на спринты, пишем код, тестируем, показываем демо заказчику и выкатываем релиз в продакшн.</t>
+          <t>Собираем требования, согласуем ТЗ и оценку, разбиваем на спринты, пишем и тестируем код, показываем демо, выкатываем релиз и передаём заказчику на поддержку.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Компания заказной разработки ПО: правда ли, что проект уходит в минус не на сложных задачах, а на бесконечных правках и часах, которых нет в смете?</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Компания заказной разработки ПО: ИИ по трекеру и истории задач прогнозирует сроки и распределяет загрузку команды, поднимает утилизацию разработчиков и держит маржу проекта в рамках оценки.</t>
         </is>
       </c>
     </row>
@@ -720,12 +756,17 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заявку, проверяем клиента, открываем расчётный счёт, подключаем эквайринг и зарплатный проект, проводим платежи и предлагаем кредитные продукты.</t>
+          <t>Принимаем заявку, проверяем клиента по требованиям комплаенса, открываем расчётный счёт, подключаем эквайринг, зарплатный проект и валютный контроль, проводим платежи, мониторим операции и предлагаем кредитные продукты.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Банк для малого бизнеса: выглядит как рост базы, но какой толк от тысяч открытых счетов, если половина пустая и не приносит ни рубля комиссий?</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Банк для малого бизнеса: ИИ по транзакционному профилю счёта подбирает нужный продукт (эквайринг, зарплатный, кредит) в момент потребности, поднимает комиссионный доход с одного счёта.</t>
         </is>
       </c>
     </row>
@@ -763,6 +804,11 @@
           <t>Языковая онлайн-школа: можно ли вырасти, если привлечение ученика стоит как три средних чека, а он бросает раньше, чем окупит первый платёж?</t>
         </is>
       </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Языковая онлайн-школа: ИИ по посещаемости, домашкам и прогрессу выявляет учеников на грани отвала и запускает триггерные касания до отмены, поднимает доходимость и LTV ученика.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -790,12 +836,17 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Закупаем зерно и молоко, настраиваем помол, готовим напитки на потоке, пробиваем чек, докупаем скоропорт и списываем нераспроданную выпечку к закрытию.</t>
+          <t>Закупаем зерно и молоко, настраиваем помол под смену, готовим напитки на потоке, предлагаем выпечку и десерт к кофе, пробиваем чек, докупаем скоропорт и списываем нераспроданное к закрытию.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Кофейня: что ломается первым, когда весь бизнес держится на утреннем часе пик — маржа на вечерних списаниях или нервы баристы в очереди?</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Кофейня: ИИ на кассе подсказывает баристе персональные допредложения к заказу и запускает акции на дневные часы, поднимает средний чек и сглаживает провал выручки после утреннего пика.</t>
         </is>
       </c>
     </row>
@@ -825,12 +876,17 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заказ, назначаем курьера, строим маршрут, забираем отправление, везём получателю, подтверждаем вручение и закрываем оплату по факту доставки.</t>
+          <t>Принимаем заказы, сортируем и консолидируем их в маршруты, назначаем курьеров, забираем отправления, доставляем получателям, при неудаче переназначаем повторную попытку и закрываем оплату по факту вручения.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Курьерская служба: где растворяется прибыль, если курьер полдня едет впустую, а неудачные попытки вручения приходится оплачивать дважды?</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Курьерская служба: ИИ строит маршруты с учётом окон доставки и вероятности недозвона, сокращает холостой пробег и повторные попытки вручения, поднимает число доставок на курьера в смену.</t>
         </is>
       </c>
     </row>
@@ -868,6 +924,11 @@
           <t>Рекрутинговое агентство: как так выходит, что вакансия закрыта, а гонорар приходится возвращать, когда нанятый кандидат уходит на испытательном сроке?</t>
         </is>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Рекрутинговое агентство: ИИ сопоставляет резюме с требованиями вакансии и ранжирует кандидатов по вероятности выхода и прохождения испытательного, поднимает долю закрытых вакансий и режет гарантийные замены.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -895,12 +956,17 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Снимаем бриф, изучаем рынок и конкурентов, разрабатываем концепции, презентуем варианты, дорабатываем выбранный и собираем брендбук с гайдлайнами.</t>
+          <t>Снимаем бриф, исследуем рынок и аудиторию, разрабатываем платформу бренда и позиционирование, придумываем нейминг и айдентику, презентуем и дорабатываем варианты, собираем брендбук с гайдлайнами.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Брендинговое агентство: куда девается маржа проекта, если он застрял на пятом круге правок, а фикс за работу давно закрыт?</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Брендинговое агентство: ИИ транскрибирует созвоны и сводит правки клиента в структурированное согласованное ТЗ, сокращает бесконечные круги правок и защищает загрузку дизайнеров и маржу проекта.</t>
         </is>
       </c>
     </row>
@@ -938,6 +1004,11 @@
           <t>Дистрибьютор продуктов питания: сколько теряет бизнес на списаниях по срокам годности и зависшей дебиторке, пока розница тянет с оплатой поставленного товара?</t>
         </is>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Дистрибьютор продуктов питания: ИИ скорит торговые точки по риску просрочки платежа и задаёт лимиты и приоритет отгрузки, сокращает зависшую дебиторку и потери на неплатежах.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -973,6 +1044,11 @@
           <t>Агентство недвижимости: что мешает сделке состояться, если показов десятки, база огромная, а клиент в итоге покупает через соседнего риелтора?</t>
         </is>
       </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Агентство недвижимости: ИИ скорит заявки по готовности к сделке и бюджету, направляет риелторов на горячих клиентов, поднимает конверсию показов в договоры и не распыляет время на пустые показы.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1008,6 +1084,11 @@
           <t>Автосервис: подъёмники заняты весь день, механики в мыле, а нормо-часы к вечеру не сходятся с кассой — так где оседает заработанное?</t>
         </is>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Автосервис: ИИ сверяет нормо-часы, списанные запчасти и кассу, выявляет аномалии и утечки по сменам и мастерам, возвращает недосчитанную выручку и сводит нормо-часы с кассой.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1035,12 +1116,17 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Формируем заказ поставщикам, принимаем и проверяем товар, выкладываем на полки, следим за ценниками, пробиваем на кассе и проводим инвентаризацию.</t>
+          <t>Заказываем товар у поставщиков, принимаем и проверяем поставку, выкладываем на полки и обновляем ценники, контролируем сроки годности, пробиваем на кассе, списываем скоропорт и проводим инвентаризацию.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Магазин у дома: куда исчезает наценка, если полки всегда полные, но списания скоропорта и недостачи на кассе тихо съедают дневную выручку?</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Магазин у дома: ИИ прогнозирует спрос по SKU и срокам годности, формирует заказ и своевременную уценку скоропорта, сокращает вечерние списания и поднимает оборачиваемость полки.</t>
         </is>
       </c>
     </row>
@@ -1070,12 +1156,17 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Принимаем устройство, проводим диагностику, называем цену, заказываем запчасть, меняем модуль, тестируем аппарат и выдаём клиенту с гарантией.</t>
+          <t>Принимаем аппарат, фиксируем в акте внешнее состояние и комплектность, диагностируем неисправность, согласуем цену до работ, заказываем деталь, меняем модуль, тестируем и выдаём клиенту с гарантией.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Сервисный центр смартфонов: сколько заказов срывается, пока клиент неделю ждёт запчасть, а рядом за углом ему чинят телефон за час?</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Сервисный центр смартфонов: ИИ прогнозирует спрос на модули и запчасти по моделям и держит ходовые на складе, убирает недельное ожидание детали и не теряет заказы, повышая загрузку мастеров.</t>
         </is>
       </c>
     </row>
@@ -1113,6 +1204,11 @@
           <t>Оптовая торговая компания: не парадокс ли — склад забит, отгрузки идут каждый день, а свободных денег нет, потому что они зависли в неликвиде?</t>
         </is>
       </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Оптовая торговая компания: ИИ по истории продаж прогнозирует спрос и планирует объёмы закупок по позициям, помечает неликвид для уценки, ускоряет оборачиваемость склада и высвобождает замороженные в товаре деньги.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1148,6 +1244,11 @@
           <t>Агентство коммерческой недвижимости: что рушит сделку на финальном шаге, когда объект найден, стороны согласны, а комиссия за полгода работы висит на волоске?</t>
         </is>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Агентство коммерческой недвижимости: ИИ сопоставляет объекты с запросами арендаторов и ранжирует сделки по вероятности закрытия, сокращает цикл сделки и снижает риск срыва на финале.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1183,6 +1284,11 @@
           <t>Частная медицинская клиника: где теряется выручка, если расписание врача в дырах от неявок, а половина пациентов не возвращается на повторный приём?</t>
         </is>
       </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Частная медицинская клиника: ИИ прогнозирует неявки и умно наполняет расписание, а триггерными напоминаниями возвращает пациентов на повторные визиты, поднимает загрузку врачей и долю дошедших назначений.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1218,6 +1324,11 @@
           <t>Управленческий консалтинг: что если ваш дорогой стратегический отчёт лёг в стол, потому что красивые слайды продать проще, чем измеримый результат на цифрах?</t>
         </is>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Управленческий консалтинг: ИИ транскрибирует интервью и воркшопы и готовит черновики отчётов и рекомендаций, поднимает утилизацию консультантов и делает результат повторяемым для повторных продаж.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1253,6 +1364,11 @@
           <t>Дистрибьютор строительных материалов: куда замораживаются деньги, когда сезон стройки закончился, а склад забит поддонами, которые до весны точно не продать?</t>
         </is>
       </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Дистрибьютор строительных материалов: ИИ прогнозирует сезонный спрос по позициям и планирует закупки под сезон, сглаживает пик и провал склада и высвобождает оборотные деньги зимой.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1288,6 +1404,11 @@
           <t>Управляющая компания арендной недвижимости: сколько съедает один месяц простоя между арендаторами, если он разом обнуляет годовую доходность объекта?</t>
         </is>
       </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Управляющая компания арендной недвижимости: ИИ скорит арендаторов по риску неплатежа и заранее сигналит о просрочках для приоритетного взыскания, поднимает собираемость и режет висящие кварталами долги.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1323,6 +1444,11 @@
           <t>Диагностический центр: отчего дорогой томограф не отбивается, если каждый его простой в пустом окне — это прямой убыток по амортизации?</t>
         </is>
       </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Диагностический центр: ИИ прогнозирует спрос на слоты и умно заполняет окна с учётом неявок и overbooking, поднимает загрузку томографа и ускоряет окупаемость дорогого оборудования.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1358,6 +1484,11 @@
           <t>Необанк: что толку от миллиона установок приложения, если добрая половина клиентов ни разу не расплатилась картой после дорогого привлечения?</t>
         </is>
       </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Необанк: ИИ ловит клиентов, засыпающих после выпуска карты, и запускает персональные триггеры на первую и регулярные операции, поднимает активацию и LTV при дорогом привлечении.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1393,6 +1524,11 @@
           <t>Дистрибьютор электроники: сколько маржи сгорает, пока партия смартфонов лежит на складе и дешевеет быстрее, чем менеджеры успевают её распродать?</t>
         </is>
       </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Дистрибьютор электроники: ИИ по скорости продаж и устареванию моделей рассчитывает своевременную уценку партии, распродаёт технику до обвала цены и удерживает маржу и оборачиваемость склада.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1428,6 +1564,11 @@
           <t>Оператор посуточной аренды: что съедает доход квартиры между заездами, если один день простоя, уборка и комиссии площадок вместе стоят дороже ночи проживания?</t>
         </is>
       </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Оператор посуточной аренды: ИИ ежедневно пересчитывает ставку под спрос, события и загрузку календаря, сокращает простой между гостями и поднимает среднюю ставку и заполняемость.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1455,12 +1596,17 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Берём биоматериал, маркируем пробирки, везём в лабораторию, ставим на анализаторы, проверяем результаты и выдаём заключение пациенту онлайн.</t>
+          <t>Берём биоматериал, маркируем и штрихкодируем пробирки, центрифугируем и сортируем пробы, ставим на анализаторы, врач валидирует результаты, выдаём заключение пациенту онлайн.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Медицинская лаборатория: где прячется себестоимость, если утром очередь на забор крови, а дорогие анализаторы полдня работают вхолостую?</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Медицинская лаборатория: ИИ прогнозирует поток проб и распределяет запись на забор по слотам, выравнивает загрузку анализаторов в течение дня, убирает утреннюю очередь и дневной простой техники, снижая себестоимость теста.</t>
         </is>
       </c>
     </row>
@@ -1498,6 +1644,11 @@
           <t>Ресторан: как так, что зал полон по выходным, а по итогам месяца ноль, если фудкост, списания и бой посуды тихо доедают всю прибыль?</t>
         </is>
       </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Ресторан: ИИ прогнозирует продажи блюд по дням недели и задаёт объём заготовок и закупок, сокращает списания в будни и удерживает фудкост при разной загрузке зала.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1525,12 +1676,17 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заявку, выезжаем к клиенту, диагностируем поломку, называем цену, заказываем запчасть, ремонтируем на месте и даём гарантию.</t>
+          <t>Принимаем заявку, выезжаем на диагностику, называем цену, при отсутствии детали заказываем её и приезжаем повторно, ремонтируем на месте, проверяем работу и даём гарантию.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Сервис ремонта бытовой техники: во сколько обходится холостой выезд, если мастер приехал через весь город, а клиент передумал чинить после названной цены?</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Сервис ремонта бытовой техники: ИИ по описанию и фото неисправности делает предварительную оценку и смету до выезда, отсекает отказников заранее и сокращает холостые выезды, поднимая маржу.</t>
         </is>
       </c>
     </row>
@@ -1560,12 +1716,17 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Покупаем участок, проектируем дом, получаем разрешения, строим корпуса, продаём квартиры через эскроу и сдаём объект дольщикам.</t>
+          <t>Покупаем участок, проектируем дом и получаем разрешения, привлекаем проектное финансирование банка, строим корпуса, продаём квартиры по ДДУ через эскроу, вводим в эксплуатацию и передаём дольщикам.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Девелопер жилой недвижимости: что опаснее — непроданные остатки в уже сданном доме или кассовый разрыв, когда стройка обгоняет темп продаж?</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Девелопер жилой недвижимости: ИИ по темпу продаж, воронке лидов и остаткам по типам квартир ежедневно корректирует цены и скидки, распродавая неликвид сданных корпусов без обвала маржи проекта.</t>
         </is>
       </c>
     </row>
@@ -1603,6 +1764,11 @@
           <t>Клиника репродуктивной медицины: почему при среднем чеке в сотни тысяч пациент отваливается ещё до пункции — на очередях, тревоге и неотвеченных звонках?</t>
         </is>
       </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Клиника репродуктивной медицины: ИИ на данных анамнеза, гормонов и снимков эмбрионов подбирает протокол стимуляции и ранжирует эмбрионы для переноса, повышая долю успешных циклов и возвраты на повторный протокол.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1638,6 +1804,11 @@
           <t>Private label бренд на маркетплейсах: куда утекает прибыль, когда оборот растёт, а вся маржа оседает в неликвиде на складе и растущей ставке хранения?</t>
         </is>
       </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Private label бренд на маркетплейсах: ИИ по истории продаж, сезонности и рекламе прогнозирует спрос на каждый SKU перед выкупом партии, снижая неликвид на складе и плату за хранение.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1673,6 +1844,11 @@
           <t>Супермаркет: сколько прибыли уезжает в мусорный бак каждый вечер, когда молочка и выпечка не проданы, а заказ на завтра уже сделан наугад?</t>
         </is>
       </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Супермаркет: ИИ по чекам, срокам годности и остаткам считает заказ скоропорта и запускает автоуценку молочки и выпечки перед истечением срока, сокращая вечерние списания и потери маржи.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1708,6 +1884,11 @@
           <t>Дистрибьютор автозапчастей: почему при полном складе клиент всё равно уходит к конкуренту — за той единственной позицией, которой не оказалось в наличии?</t>
         </is>
       </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Дистрибьютор автозапчастей: ИИ по кросс-номерам, VIN и каталогам мгновенно подбирает точный аналог, когда запрошенной позиции нет в наличии, удерживая заявку сервиса вместо ухода к конкуренту.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1743,6 +1924,11 @@
           <t>Косметологическая клиника: куда утекает выручка, когда дорогой аппарат окупается годами, а клиент делает одну процедуру и не возвращается на курс?</t>
         </is>
       </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Косметологическая клиника: ИИ по истории процедур и типу кожи клиента рекомендует следующий шаг курса и домашний уход, превращая разовые визиты в курсы и поднимая средний чек и LTV.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1778,6 +1964,11 @@
           <t>Платёжный агрегатор: сколько оборота теряется на отклонённых транзакциях, которые были честными, но не прошли слишком грубый фильтр против мошенников?</t>
         </is>
       </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Платёжный агрегатор: ИИ-антифрод оценивает каждую транзакцию по поведению и устройству, отделяя честные платежи от мошеннических, снижая долю ложных отказов и возвращая мерчантам потерянный оборот.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1813,6 +2004,11 @@
           <t>Пиццерия: почему при полной посадке в пятницу месяц всё равно уходит в ноль — из-за простоя печей в будни и вечно дорожающего сыра?</t>
         </is>
       </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Пиццерия: ИИ прогнозирует спрос по часам и дням и запускает адресные будние акции и комбо, загружая простаивающие вне пятничного пика печи и выравнивая маржу заказа.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1848,6 +2044,11 @@
           <t>Дистрибьютор медицинских товаров: куда девается прибыль, когда тендер выигран, но отсрочка клиники на 90 дней и списанная просрочка съедают всю наценку?</t>
         </is>
       </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Дистрибьютор медицинских товаров: ИИ по истории оплат, тендерам и финансовым признакам клиник скорит риск просрочки перед отгрузкой в отсрочку, снижая кассовые разрывы и потери на просроченной дебиторке.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1883,6 +2084,11 @@
           <t>Компания по строительству загородных домов: почему прибыльный на бумаге дом уходит в убыток — на переделках, простое бригад и подорожавших к середине стройки материалах?</t>
         </is>
       </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Компания по строительству загородных домов: ИИ по проекту, ценам поставщиков и нормам расхода собирает смету и спецификацию за минуты, снижая ошибки расчёта и переделки, съедающие маржу.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1918,6 +2124,11 @@
           <t>Химчистка: сколько прибыли теряется на одной испорченной шубе, когда компенсация клиенту перекрывает выручку за десятки обычных заказов?</t>
         </is>
       </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Химчистка: компьютерное зрение по фото изделия при приёмке определяет тип ткани, пятна и риск порчи, подсказывая безопасный режим и фиксируя дефекты, что снижает претензии и компенсации за порчу.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1953,6 +2164,11 @@
           <t>Консалтинг по продажам: почему клиент платит за рост выручки, но через три месяца отдел откатывается к старым привычкам, а виноватым остаётся консультант?</t>
         </is>
       </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Консалтинг по продажам: ИИ анализирует все звонки и переписку отдела клиента, оценивает соблюдение скриптов и выявляет провалы конверсии, удерживая результат после ухода консультанта и убирая откат к старым привычкам.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1988,6 +2204,11 @@
           <t>Дистрибьютор косметики: куда уходит наценка, когда сеть требует отсрочку и ретробонус, а сезонная коллекция уже висит на складе мёртвым грузом?</t>
         </is>
       </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Дистрибьютор косметики: ИИ по остаткам, срокам годности и продажам сетей рассчитывает цены и глубину скидок для сезонных коллекций, распродавая короткосрочный товар до списания и защищая наценку.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2023,6 +2244,11 @@
           <t>Архитектурное бюро: почему гонорар за проект тает в бесконечных правках, которые заказчик считает мелочью, а бюро — неоплаченными переделками?</t>
         </is>
       </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Архитектурное бюро: генеративный ИИ по брифу и участку выдаёт несколько вариантов концепции и визуализаций за часы вместо недель, ускоряя согласование с заказчиком и сокращая неоплаченные переделки эскизов.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2058,6 +2284,11 @@
           <t>Магазин одежды: сколько прибыли лежит мёртвым грузом на вешалках, когда популярных размеров уже нет, а весь неликвид ждёт скидки минус семьдесят?</t>
         </is>
       </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Магазин одежды: ИИ по продажам, размерной сетке и погоде прогнозирует спрос и вовремя дозаказывает ходовые размеры, сокращая вымывание бестселлеров и остатки, которые уходят в сезонную уценку.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2065,7 +2296,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Executive search агентство</t>
+          <t>Детский лагерь</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2075,22 +2306,27 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Фикс + success fee</t>
+          <t>Оплата за смену</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Executive search агентство: как масштабировать закрытие вакансий топов и защитить success fee, если весь результат держится на личной сети хедхантера?</t>
+          <t>Детский лагерь: как заполнить все смены сезона и удержать вожатых, если весь годовой доход спрессован в три летних месяца?</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Снимаем требования к позиции, строим карту рынка и лонг-лист кандидатов, выходим на пассивных топов, проводим интервью и оценку, представляем шорт-лист, сопровождаем оффер и выход.</t>
+          <t>Мы набираем детей на смены, готовим программу и корпуса, обучаем и распределяем вожатых, кормим и расселяем отряды, ведём кружки и активности, следим за безопасностью и держим связь с родителями.</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Executive search агентство: почему полгода работы над вакансией сгорают дотла, когда финальный кандидат в последний момент принимает контроффер?</t>
+          <t>Детский лагерь: почему полная смена не значит прибыль, если недобор одного отряда обнуляет заработок за всё короткое лето?</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Детский лагерь: ИИ оптимизирует рекламные бюджеты и таргетинг по каналам и сменам, дозаполняя недобранные отряды и снижая стоимость заявки родителя, чтобы каждая смена сезона выходила в плюс.</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2336,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Дистрибьютор офисных товаров</t>
+          <t>Ростерия (обжарка кофе)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2110,22 +2346,27 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Оптовая маржа</t>
+          <t>Производство + продажи</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Дистрибьютор офисных товаров: как удержать оптовую маржу на копеечных позициях, если корпоративные клиенты выбивают отсрочку, а логистика мелких заказов съедает наценку?</t>
+          <t>Ростерия (обжарка кофе): как балансировать объём обжарки под опт и розницу, чтобы зерно не залёживалось и не теряло свежесть?</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Держим широкий каталог канцелярии и расходников, принимаем заявки компаний, комплектуем сборные заказы, доставляем в офисы, выставляем счета с отсрочкой, обрабатываем возвраты и допоставки.</t>
+          <t>Мы закупаем зелёное зерно, обжариваем партиями по профилям, дегустируем и отсеиваем брак, фасуем с датой обжарки, отгружаем оптовым кофейням и продаём в розницу, отслеживая свежесть остатков.</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Дистрибьютор офисных товаров: куда утекает прибыль, когда клиент заказывает пачку бумаги и три ручки, а доставка через весь город стоит дороже самой маржи?</t>
+          <t>Ростерия (обжарка кофе): сколько прибыли сгорает вместе с зерном, если обжаренная партия теряет цену с каждым днём на полке?</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Ростерия (обжарка кофе): ИИ по заказам опта, рознице и свежести остатков планирует объём и график обжарки по профилям, сокращая залежавшееся зерно и потери цены на полке.</t>
         </is>
       </c>
     </row>
@@ -2163,6 +2404,11 @@
           <t>Дизайн-студия интерьеров: почему красивый проект уходит в минус, когда заказчик двадцатый раз меняет диван, а часы дизайнера никто не оплачивает?</t>
         </is>
       </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Дизайн-студия интерьеров: ИИ-конфигуратор в реальном времени показывает заказчику фотореалистичные варианты мебели и материалов в его планировке, сокращая бесконечные правки и неоплаченные часы дизайнера.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2198,6 +2444,11 @@
           <t>Психологический центр: куда утекает выручка, когда клиент бросает терапию после третьей сессии, а окно в расписании психолога так и остаётся пустым?</t>
         </is>
       </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Психологический центр: ИИ по первичному запросу и профилям специалистов точнее подбирает психолога под клиента, снижая отсев после двух-трёх сессий и заполняя простаивающие окна в расписании.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2233,6 +2484,11 @@
           <t>Fulfillment-оператор: почему при тысячах отгрузок в день оператор еле выходит в ноль — на ошибках сборки, возвратах и простое склада между пиками?</t>
         </is>
       </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Fulfillment-оператор: ИИ по потоку заказов и календарю площадок прогнозирует почасовую нагрузку и планирует смены сборщиков, убирая простой между пиками и переработки в часы отгрузок.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2268,6 +2524,11 @@
           <t>Производитель одежды: куда уходит прибыль, когда цех то стоит без загрузки, то срывает сроки, а рулоны дорогой ткани лежат в остатках раскроя?</t>
         </is>
       </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Производитель одежды: ИИ планирует загрузку швейного цеха и очередность раскроя по заказам и срокам, сглаживая простои и авралы и поднимая утилизацию оборудования между коллекциями.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2303,6 +2564,11 @@
           <t>Производитель кухонь на заказ: сколько маржи сгорает на одной ошибке в замере, когда готовый фасад не встаёт по месту и весь модуль идёт в переделку?</t>
         </is>
       </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Производитель кухонь на заказ: ИИ по замеру автоматически строит спецификацию, карту раскроя и проверяет коллизии размеров до распила, сокращая ошибки и дорогие переделки фасадов и модулей.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2338,6 +2604,11 @@
           <t>Продавец одежды на маркетплейсах: правда ли, что каждый второй заказ возвращается — и вся прибыль тонет в обратной логистике и помятом при примерке товаре?</t>
         </is>
       </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Продавец одежды на маркетплейсах: ИИ по параметрам покупателя и отзывам о посадке рекомендует точный размер на карточке, снижая долю возвратов и обратную логистику, съедающую маржу.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2373,6 +2644,11 @@
           <t>Оператор денежных переводов: куда утекает комиссия, когда клиент сравнивает курс за секунду и уходит к тому, у кого дешевле на полпроцента?</t>
         </is>
       </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Оператор денежных переводов: ИИ по коридорам, объёму и чувствительности сегмента динамически подбирает курс и комиссию, удерживая клиента, сравнивающего цену за секунду, без обвала и без того тонкой маржи.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2408,6 +2684,11 @@
           <t>Магазин косметики: сколько прибыли уходит в тестеры и просрочку, пока полка забита ассортиментом, а покупают одни и те же десять позиций?</t>
         </is>
       </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Магазин косметики: ИИ по продажам и оборачиваемости чистит ассортимент, оптимизирует выкладку и заказ, сокращая просрочку и лишние тестеры и высвобождая полку под реально покупаемые позиции.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2415,7 +2696,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Мебельная студия на заказ</t>
+          <t>Компания по натяжным потолкам</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2430,17 +2711,22 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Мебельная студия на заказ: как ускорить путь от эскиза до готового изделия и держать маржу, если каждый шкаф-купе считается заново вручную?</t>
+          <t>Компания по натяжным потолкам: как уплотнить график монтажных бригад и поднять маржу, если замер и установка часто идут одним выездом?</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Обсуждаем задачу и делаем замер, проектируем изделие и считаем материалы, согласуем с клиентом, заказываем распил и фурнитуру, собираем в цеху, доставляем и устанавливаем.</t>
+          <t>Мы принимаем заявку, выезжаем на замер, считаем смету и материал, кроим полотно, монтируем каркас и натягиваем потолок за один выезд, ставим светильники и сдаём работу заказчику.</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Мебельная студия на заказ: почему прибыль тает между замером и монтажом — на ручном пересчёте спецификаций и переделках из-за неучтённого миллиметра?</t>
+          <t>Компания по натяжным потолкам: где прячется прибыль, если за целый день бригада натягивает один потолок, а половину смены съедают дорога и замеры?</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Компания по натяжным потолкам: ИИ группирует замеры и монтажи по географии и строит маршруты бригад, уплотняя график выездов и сокращая время на дорогу, что поднимает число объектов в день.</t>
         </is>
       </c>
     </row>
@@ -2478,6 +2764,11 @@
           <t>Телемедицинский сервис: куда утекает выручка, когда пациент задал один вопрос, закрыл приложение и записался к живому врачу вместо повторной консультации?</t>
         </is>
       </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Телемедицинский сервис: ИИ выявляет пациентов с риском не вернуться и запускает персональные follow-up по итогам консультации, поднимая долю повторных обращений и загрузку врачей платформы.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2513,6 +2804,11 @@
           <t>Экспедиторская компания: сколько ставки съедает порожний обратный рейс, когда машина едет назад пустой, а водитель всё равно стоит на погрузке полдня?</t>
         </is>
       </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Экспедиторская компания: ИИ подбирает обратную загрузку и строит маршруты под заявки, сокращая порожние пробеги и простои на погрузке, что поднимает маржу на рейсе.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -2548,6 +2844,11 @@
           <t>Агентство временного персонала: куда утекает маржа, когда треть смены не выходит, клиент штрафует за срыв, а замену приходится искать за час до открытия?</t>
         </is>
       </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Агентство временного персонала: ИИ скорит надёжность работников по истории выходов и мгновенно подбирает замену из пула под срочную заявку, снижая срывы смен и штрафы клиентов.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2583,6 +2884,11 @@
           <t>Производитель обуви: куда уходит прибыль, когда ходовые размеры распроданы, а склад забит крайними — которые не берут даже со скидкой?</t>
         </is>
       </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Производитель обуви: ИИ по продажам и размерной сетке прогнозирует спрос и план тиража по размерам, сокращая склад неходовых крайних размеров и вымывание популярных пар.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2618,6 +2924,11 @@
           <t>Суши-доставка: почему при полном потоке в пятницу прибыль тает — между комиссией агрегатора, дорогой рыбой и роллами, списанными к концу смены?</t>
         </is>
       </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Суши-доставка: прогноз спроса на роллы по часам и дням из истории заказов агрегаторов задаёт объём нарезки рыбы и заготовок, сокращая списания к концу смены и поднимая маржу заказа.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -2653,6 +2964,11 @@
           <t>Прачечная самообслуживания: почему барабаны крутятся на всю мощность вечером, но полдня стоят пустыми и всё это время съедают аренду?</t>
         </is>
       </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Прачечная самообслуживания: динамическое ценообразование циклов по времени суток — дневные скидки в приложении из данных загрузки машин заполняют простой между вечерними пиками и поднимают выручку с барабана.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2688,6 +3004,11 @@
           <t>Продавец косметики на маркетплейсах: куда утекает прибыль, если выкуп растёт, а остатки крема надо продать раньше, чем закончится срок годности?</t>
         </is>
       </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Продавец косметики на маркетплейсах: прогноз спроса по SKU и сроку годности из продаж и остатков площадки задаёт размер партий закупки, снижая просрочку и замороженные в неликвиде деньги.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -2715,12 +3036,17 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Выезжаем на замер, просчитываем смету, распиливаем ЛДСП, клеим кромку, ставим фурнитуру, собираем корпус в цеху и монтируем у клиента.</t>
+          <t>Разрабатываем модельный ряд, закупаем ЛДСП и фурнитуру, распиливаем и кромим детали, сверлим присадку и собираем корпуса партиями, упаковываем в плоские короба, храним на складе и отгружаем в розницу и опт.</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Производитель мебели: правда ли, что прибыль съедает не сырьё, а один неверный замер, из-за которого лист уходит в брак и переделку?</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Производитель мебели: ИИ по индивидуальным размерам заказа автоматически формирует спецификацию, карту раскроя и смету, убирая ошибки ручного расчёта и брак листа ЛДСП из-за неверного замера.</t>
         </is>
       </c>
     </row>
@@ -2758,6 +3084,11 @@
           <t>Компания по установке окон: что ломается первым, когда летом заказов больше, чем монтажников, а зимой бригады сидят без выработки?</t>
         </is>
       </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Компания по установке окон: прогноз сезонного потока заявок по годам и погоде планирует загрузку бригад заранее, сглаживая летний перегруз и зимний простой без потери выработки.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2785,12 +3116,17 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заявку, выезжаем на замер, штробим стену, прокладываем трассу, вешаем блоки, вакуумируем систему, заправляем фреоном и запускаем сплит-систему.</t>
+          <t>Принимаем заявку, выезжаем на замер, бурим отверстие под трассу, вешаем внутренний и внешний блоки, прокладываем и вакуумируем магистраль, запускаем и проверяем сплит-систему.</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
           <t>Компания по монтажу кондиционеров: сколько выручки утекает в жару, когда телефон разрывается, а свободных бригад на монтаж уже нет?</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Компания по монтажу кондиционеров: ИИ строит плотные маршруты и расписание бригад в пик, вмещая больше монтажей за смену и снимая максимум выручки короткого сезона.</t>
         </is>
       </c>
     </row>
@@ -2828,6 +3164,11 @@
           <t>Грузоперевозочная компания: куда уезжает прибыль, если фура едет туда с грузом, а обратно — с воздухом и полным баком солярки?</t>
         </is>
       </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Грузоперевозочная компания: ИИ подбирает попутную загрузку под обратный маршрут из заявок и бирж грузов, сокращая порожние пробеги и расход солярки и поднимая доходность рейса.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -2863,6 +3204,11 @@
           <t>Производитель матрасов: почему товар с хорошей наценкой всё равно балансирует у нуля, когда склад и доставка съедают её своим объёмом?</t>
         </is>
       </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Производитель матрасов: ИИ консолидирует доставки габарита в общие рейсы и строит маршруты по адресам заказов, снижая долю логистики и хранения в цене каждого матраса.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -2898,6 +3244,11 @@
           <t>Ветеринарная клиника: где теряются деньги, когда врач занят одним тяжёлым случаем, а очередь из плановых прививок расходится по конкурентам?</t>
         </is>
       </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Ветеринарная клиника: ИИ по картам питомцев напоминает о плановых прививках, дегельминтизации и повторных приёмах точно в срок, возвращая владельцев вместо ухода к конкурентам.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -2925,12 +3276,17 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Аудируем бизнес клиента, упаковываем франшизу, считаем финмодель, пишем стандарты, готовим презентацию, находим покупателей лотов и сопровождаем первые запуски.</t>
+          <t>Аудируем бизнес клиента, упаковываем стандарты и финмодель, регистрируем товарный знак и готовим договор концессии, собираем продающую презентацию, находим покупателей лотов и сопровождаем первые запуски.</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
           <t>Консалтинг по франчайзингу: что скрывается за красивой упаковкой, если франшизу продали, паушалку взяли, а франчайзи прогорел через полгода?</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Консалтинг по франчайзингу: RAG-ассистент по стандартам и финмодели отвечает франчайзи на вопросы запуска из базы регламентов, снижая долю прогоревших точек и защищая поток роялти.</t>
         </is>
       </c>
     </row>
@@ -2960,12 +3316,17 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Ищем ходовые позиции, закупаем партию, фотографируем, заполняем карточки, отгружаем на склад площадки, следим за остатками и обрабатываем возвраты.</t>
+          <t>Ищем ходовые позиции, закупаем партию, снимаем фото и заполняем карточки, отгружаем на склад площадки, продвигаем рекламой, следим за остатками и стоимостью хранения габарита, обрабатываем возвраты.</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Продавец товаров для дома на маркетплейсах: почему объёмный товар с виду продаётся, а за его хранение площадка списывает больше, чем он приносит?</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Продавец товаров для дома на маркетплейсах: ИИ считает оборачиваемость и стоимость хранения по каждому габаритному SKU, отсекая позиции, где склад площадки съедает наценку быстрее, чем товар продаётся.</t>
         </is>
       </c>
     </row>
@@ -3003,6 +3364,11 @@
           <t>Производитель окон и дверей: что съедает маржу, если дилеры давят на цену, а цех то стоит без загрузки, то не успевает в сезон?</t>
         </is>
       </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Производитель окон и дверей: прогноз заказов дилеров по сезону и истории отгрузок выравнивает план производства и закупку профиля, убирая простой цеха в межсезонье и авралы в пик.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3038,6 +3404,11 @@
           <t>Магазин электроники: правда ли, что смартфон на витрине почти не приносит прибыли, а вся маржа прячется в чехле и страховке рядом с ним?</t>
         </is>
       </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>Магазин электроники: ИИ по модели в чеке рекомендует продавцу релевантные аксессуары, гарантию и сервис, поднимая долю высокомаржинальных допов и средний чек там, где на самой технике наценка минимальна.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3065,12 +3436,17 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заказ из агрегатора, готовим блюдо по чек-листу, собираем и упаковываем, передаём курьеру, держим рейтинг и следим за себестоимостью порции.</t>
+          <t>Закупаем продукты, готовим блюда нескольких виртуальных брендов по чек-листам, принимаем заказы из агрегаторов, собираем и упаковываем, передаём курьерам, держим скорость и рейтинг, следим за себестоимостью порции.</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
           <t>Dark kitchen: куда исчезает прибыль кухни без зала, если агрегатор забирает четверть чека, а лишняя минута сборки роняет рейтинг?</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Dark kitchen: ИИ разбирает отзывы и оценки из агрегаторов по каждому виртуальному бренду, вычленяя причины падения рейтинга — долгую сборку, ошибки набора — чтобы удерживать рейтинг и поток заказов.</t>
         </is>
       </c>
     </row>
@@ -3108,6 +3484,11 @@
           <t>Ателье: почему мастер весь день подшивает брюки за копейки, а очередь на дорогой пошив стоит, потому что руки заняты мелочью?</t>
         </is>
       </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Ателье: ИИ при приёме оценивает доходность и сложность каждого заказа и приоритизирует в расписании мастера дорогой пошив и срочные, чтобы время не уходило на копеечную подгонку.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3143,6 +3524,11 @@
           <t>Производитель строительных материалов: что происходит с деньгами, когда летом линия не успевает, а зимой склад забит непроданными паллетами?</t>
         </is>
       </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Производитель строительных материалов: динамическое ценообразование с зимними скидками дилерам по данным спроса и складских остатков разгружает забитый межсезонный склад и держит линию загруженной круглый год.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3178,6 +3564,11 @@
           <t>Электромонтажная компания: что остаётся от прибыли объекта, если смету считали на глаз, а кабеля и работы по факту ушло в полтора раза больше?</t>
         </is>
       </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Электромонтажная компания: ИИ по проекту и плану помещения автоматически считает смету — метраж кабеля, число точек, работы — сближая план с фактом и убирая убыток от недосчитанных материалов и переделок.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3213,6 +3604,11 @@
           <t>HR-аутсорсинг: что мешает расти, если новых клиентов берёшь легко, а каждый тонет в трудовых книжках, приказах и оформлении вручную?</t>
         </is>
       </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>HR-аутсорсинг: ИИ распознаёт паспорта, СНИЛС и трудовые и автозаполняет приказы и кадровые формы, убирая ручной ввод, чтобы брать больше клиентов на абонентку без роста штата.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3248,6 +3644,11 @@
           <t>Сервис интернет-эквайринга: сколько зарабатываешь на доле процента, если один спорный платёж и чарджбек съедают прибыль с сотни успешных?</t>
         </is>
       </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Сервис интернет-эквайринга: ИИ-антифрод по паттернам транзакций мерчанта в реальном времени помечает аномальные платежи и вероятные чарджбеки, сокращая потери и споры, съедающие тонкую комиссию.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -3283,6 +3684,11 @@
           <t>Бухгалтерский аутсорсинг: как выходит, что абонентка фиксированная, а клиент с горой неразобранных чеков и актов уводит вас в глубокий минус?</t>
         </is>
       </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>Бухгалтерский аутсорсинг: ИИ распознаёт первичку — счета, акты, накладные — и разносит по учёту с автосверкой контрагентов, освобождая время бухгалтера на новых клиентов абонентки.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -3310,12 +3716,17 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Ведём запись, встречаем клиента, выполняем услугу, предлагаем уход и допроцедуры, берём оплату, зовём на повтор и докупаем расходники.</t>
+          <t>Ведём запись и подбираем мастера, встречаем клиента, стрижём, красим и укладываем, предлагаем уход и допуслуги, берём оплату, зовём на повтор и докупаем расходники.</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
           <t>Салон красоты: сколько теряет салон на пустых окнах между записями, за которые аренда капает так же, как за занятые кресла?</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Салон красоты: ИИ дозаполняет пустые окна между записями, предлагая клиентам из базы удобный слот и короткую услугу, поднимая утилизацию кресел и выручку с арендуемого места.</t>
         </is>
       </c>
     </row>
@@ -3345,12 +3756,17 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заявку, оформляем документы, строим мультимодальный маршрут, проходим таможню через брокера, ведём груз через границы и передаём получателю.</t>
+          <t>Принимаем заявку, подбираем перевозчика и букируем фрахт, строим мультимодальный маршрут, оформляем документы и страховку, проходим таможню через брокера, ведём груз через границы и передаём получателю.</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
           <t>Компания по международным перевозкам: сколько стоит один день простоя на таможне, если фура ждёт бумагу, а клиент считает срок, а не километры?</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>Компания по международным перевозкам: ИИ извлекает данные из инвойсов, упаковочных листов и CMR и готовит пакет к таможне, сокращая простой фуры на границе из-за документов.</t>
         </is>
       </c>
     </row>
@@ -3388,6 +3804,11 @@
           <t>Фотоателье: почему очередь за фото на паспорт есть всегда, а денег с неё мало, пока дорогая печать и портреты простаивают?</t>
         </is>
       </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Фотоателье: ИИ-ретушь и генерация деловых портретов и стилизованных фото из одного снимка превращают дешёвую съёмку на документы в апселл, поднимая средний чек и загружая простаивающую печать.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -3423,6 +3844,11 @@
           <t>Мебельный салон: что уводит покупателя, если диван понравился, но ждать его с фабрики месяц, а решение он принимает сегодня?</t>
         </is>
       </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Мебельный салон: 3D-конфигуратор показывает выбранный диван в нужной ткани и в интерьере клиента прямо в шоуруме, удерживая решение здесь и сейчас, пока фабрика делает заказ недели.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -3458,6 +3884,11 @@
           <t>Производитель упаковки: куда уходит прибыль на маленьком заказе, если приладка машины и новый штамп стоят как половина всего тиража?</t>
         </is>
       </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Производитель упаковки: ИИ автоматически рассчитывает цену заказа с учётом приладки, стоимости штампа и раскроя картона, чтобы мелкие тиражи не уходили в минус, а КП считалось за минуты.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -3493,6 +3924,11 @@
           <t>Лизинговая компания: чем оборачивается растущий портфель, если один клиент перестал платить, а изъятый актив стоит уже вдвое дешевле?</t>
         </is>
       </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Лизинговая компания: риск-скоринг заявителя по финансам, отрасли и ликвидности предмета лизинга отсекает сделки с высокой вероятностью просрочки, снижая долю дефолтов и потери на перепродаже изъятого.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -3528,6 +3964,11 @@
           <t>Интернет-магазин электроники: во что превращается прибыль заказа, если покупатель сравнил цену до копейки, а потом ещё и вернул товар после доставки?</t>
         </is>
       </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-магазин электроники: ИИ ловит брошенные корзины и предсказывает уходящих покупателей, запуская триггерные письма и точечную скидку, чтобы вернуть заказ на тонкой марже без сплошных распродаж.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -3563,6 +4004,11 @@
           <t>Зарплатный аутсорсинг: почему абонентка за сотрудника кажется прибыльной, пока в конце месяца все клиенты требуют расчёт в один и тот же день?</t>
         </is>
       </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Зарплатный аутсорсинг: ИИ прогнозирует пик расчётов к концу месяца по числу клиентов и сотрудников и распределяет нагрузку расчётчиков заранее, чтобы уложиться в сроки выплат без раздувания штата.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -3598,6 +4044,11 @@
           <t>Типография: куда девается прибыль, если печатная машина час крутится на приладке ради тиража, который потом печатается за десять минут?</t>
         </is>
       </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>Типография: ИИ группирует заказы по формату, бумаге и краске и строит очередь печати так, чтобы сократить число приладок между мелкими тиражами и поднять загрузку машин.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -3633,6 +4084,11 @@
           <t>Сантехническая компания: почему аварийные вызовы идут потоком, а прибыли мало, если бригада тушит потопы вместо дорогих плановых монтажей?</t>
         </is>
       </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>Сантехническая компания: ИИ по данным аварийного выезда — возраст труб, состояние разводки — подсказывает мастеру плановую замену и КП на монтаж, превращая дешёвый вызов в дорогой заказ.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -3668,6 +4124,11 @@
           <t>Пекарня: сколько прибыли уходит в мусорный бак каждый вечер, когда утренний ажиотаж схлынул, а полки всё ещё полны нераспроданной выпечки?</t>
         </is>
       </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>Пекарня: прогноз почасового спроса по чекам за 12 месяцев и погоде задаёт размер утренних и дневных партий, срезая вечерние списания на 25–35% и поднимая маржу.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -3703,6 +4164,11 @@
           <t>Барбершоп: почему при полной записи прибыль тает, а «окна» между клиентами и простои в будни съедают половину рабочей смены?</t>
         </is>
       </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>Барбершоп: алгоритм уплотняет запись по истории слотов и длительности услуг мастеров, закрывая будние окна между клиентами и поднимая утилизацию кресла с 60% до 80%.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -3738,6 +4204,11 @@
           <t>Производитель наружной рекламы: куда утекает маржа, если цех загружен, а между замером, правками макета и монтажом проходят недели?</t>
         </is>
       </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>Производитель наружной рекламы: генеративный ИИ по фото объекта и брифу собирает 3–4 варианта макета вывески за минуты, сокращая круг правок и срок от замера до монтажа на неделю.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -3765,12 +4236,17 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Собираем первичку клиента, сводим управленческий учёт, считаем P&amp;L и кэшфлоу, ищем кассовые разрывы, готовим отчёт и созваниваемся с собственником.</t>
+          <t>Собираем данные из учёта клиента, сводим управленческий отчёт с P&amp;L и кэшфлоу, строим бюджет и платёжный календарь, находим кассовые разрывы и точки роста, защищаем решения перед собственником.</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
           <t>Финансовый директор на аутсорсе: почему эксперт продаёт стратегию, а по факту половину месяца сводит чужие таблицы вручную?</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>Финансовый директор на аутсорсе: ИИ распознаёт выписки, счета и оборотки клиента и автоматически сводит P&amp;L и кэшфлоу, освобождая до половины месяца на новых абонентов.</t>
         </is>
       </c>
     </row>
@@ -3800,12 +4276,17 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>Верстаем расписание сеансов, продаём билеты онлайн и в кассе, отпускаем попкорн и напитки в баре, крутим рекламу перед фильмом и убираем залы.</t>
+          <t>Бронируем прокатные копии у дистрибьюторов, верстаем расписание сеансов, продаём билеты онлайн и в кассе, отпускаем попкорн и напитки в баре, крутим рекламу перед показом и убираем залы.</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
           <t>Кинотеатр: правда ли, что пустой дневной сеанс и очередь за попкорном, не успевшая до старта фильма, — это одна и та же дыра в кассе?</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>Кинотеатр: динамическое ценообразование билетов по заполняемости, дню и релизу поднимает цену вечерних сеансов и распродаёт пустые дневные, увеличивая выручку с кресла на 10–15%.</t>
         </is>
       </c>
     </row>
@@ -3835,12 +4316,17 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Наполняем карточки с размерами, консультируем по замеру, принимаем заказ, везём со склада, поднимаем и собираем на месте, отрабатываем возвраты.</t>
+          <t>Наполняем карточки с размерами и фото, помогаем подобрать габариты, принимаем заказ, везём со склада или от фабрики, поднимаем и собираем на месте, отрабатываем возвраты крупногабарита.</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
           <t>Интернет-магазин мебели: куда исчезает прибыль, когда корзину бросают на «уточните размеры», а привезённый шкаф не влезает в лифт?</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-магазин мебели: AR-конфигуратор ставит диван по реальным габаритам в интерьер клиента, снижая брошенные на «уточните размеры» корзины и возвраты крупногабарита на 20–30%.</t>
         </is>
       </c>
     </row>
@@ -3878,6 +4364,11 @@
           <t>Металлообрабатывающее предприятие: почему при загруженных станках цех уходит в минус, если переналадка и просчёт в смете дороже самой детали?</t>
         </is>
       </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>Металлообрабатывающее предприятие: ИИ по чертежу и норме времени считает себестоимость детали с учётом переналадки и металла, ускоряя смету и убирая просчёты, что держит маржу заказа.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -3913,6 +4404,11 @@
           <t>Клининговая компания: куда утекает прибыль, если бригада выехала на объект, а половина дня ушла на дорогу, простой и переделку?</t>
         </is>
       </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>Клининговая компания: ИИ строит маршруты и графики бригад по адресам, площадям и пробкам, срезая время в дороге и простой на 20–30% и повышая выработку с бригады.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -3940,12 +4436,17 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Закупаем ходовые позиции, храним на складе, консультируем по объёму, пробиваем на кассе, грузим и организуем доставку клиенту на объект.</t>
+          <t>Закупаем ходовые позиции, храним на складе, рассчитываем материалы под смету клиента, консультируем и пробиваем на кассе, грузим и доставляем на объект, следим за остатками ходового и неликвидом.</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
           <t>Магазин строительных материалов: почему выручка есть, а денег нет, если ходовой цемент кончился, а неликвид пылится на паллетах полгода?</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>Магазин строительных материалов: прогноз спроса по сезону и истории продаж по каждой позиции задаёт закупку, сокращая неликвид на паллетах и вымывание ходового цемента из наличия.</t>
         </is>
       </c>
     </row>
@@ -3983,6 +4484,11 @@
           <t>Факторинговая компания: где прячется убыток, если комиссия капнула сегодня, а один просроченный дебитор перечёркивает маржу с десятка сделок?</t>
         </is>
       </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>Факторинговая компания: риск-скоринг дебиторов по платёжной дисциплине, отраслевым и открытым данным задаёт лимит под каждую поставку, наращивая портфель без роста доли просроченных платежей.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -4018,6 +4524,11 @@
           <t>Деревообрабатывающее предприятие: почему кубометр куплен целиком, а денег приносит только половина, если брак сушки и опилки списываются в ноль?</t>
         </is>
       </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>Деревообрабатывающее предприятие: ИИ по влажности, породе и режиму сушки прогнозирует выход годного и сорт партии, снижая брак сушки и поднимая выход товарной доски из кубометра.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -4053,6 +4564,11 @@
           <t>Юридическая фирма для бизнеса: куда утекает маржа, когда партнёр с высокой ставкой полдня правит шаблонный договор вместо сложного дела?</t>
         </is>
       </c>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>Юридическая фирма для бизнеса: ИИ по параметрам сделки собирает черновики типовых договоров и претензий из шаблонов, снимая рутину с дорогих юристов и высвобождая их на сложные дела.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -4088,6 +4604,11 @@
           <t>Кондитерская: почему предновогодний вал заказов не спасает год, если летом витрина списывается, а декор и ручной труд не заложены в цену?</t>
         </is>
       </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>Кондитерская: ИИ по истории витринных продаж и сезону планирует ассортимент и объём выкладки на день, срезая списание скоропорта и подсказывая цену заказных тортов с учётом декора.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -4115,12 +4636,17 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Находим специалистов, проверяем стек, продаём клиенту на проект по ставке, оформляем, ведём тайм-шиты, выставляем счёт и платим зарплату.</t>
+          <t>Находим специалистов, проверяем стек, продаём клиенту на проект по ставке, проводим собеседование у заказчика, оформляем, управляем загрузкой и заменами, ведём тайм-шиты, выставляем счёт и платим зарплату.</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
           <t>Аутстаффинговая IT-компания: куда исчезает прибыль, если один разработчик на бенче и две задержки замен съедают маржу с целой команды?</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>Аутстаффинговая IT-компания: ИИ сопоставляет резюме и стек специалистов с бенча с запросами клиентов, ускоряя замены и сокращая простой на бенче, что удерживает маржу команды.</t>
         </is>
       </c>
     </row>
@@ -4158,6 +4684,11 @@
           <t>Студия маникюра: почему при плотной записи касса не растёт, если между клиентами зияют окна, а любимый мастер уводит базу в свой директ?</t>
         </is>
       </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>Студия маникюра: ИИ по истории визитов клиента рекомендует мастеру релевантные допуслуги — педикюр, уход, дизайн, — поднимая средний чек на 15–20% без давления на гостя.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -4193,6 +4724,11 @@
           <t>Таможенный брокер: правда ли, что одна ошибка в коде ТН ВЭД или задержка выпуска сжигает комиссию сразу с нескольких контрактов?</t>
         </is>
       </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>Таможенный брокер: ИИ извлекает данные из инвойсов и упаковочных листов и предлагает код ТН ВЭД с обоснованием, ускоряя оформление деклараций и снижая риск ошибки и штрафа.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -4228,6 +4764,11 @@
           <t>Сервис бытового ремонта: куда утекает прибыль, если мастер полдня в пробках, а клиент отказывается от ремонта уже после платного выезда?</t>
         </is>
       </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>Сервис бытового ремонта: ИИ по фото и описанию поломки предварительно ставит диагноз, подбирает запчасть и цену до выезда, срезая напрасные выезды и отказы после платной диагностики.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -4263,6 +4804,11 @@
           <t>Детский развлекательный центр: почему аренда съедает выручку, если по будням залы пустуют, а вся касса втискивается в два выходных дня?</t>
         </is>
       </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>Детский развлекательный центр: динамические цены и промо на будни по прогнозу посещаемости заполняют пустые дневные часы, выравнивая выручку между буднями и перегруженными выходными.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -4270,7 +4816,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Копировальный центр</t>
+          <t>Свадебное агентство</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -4280,22 +4826,27 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Оплата за услугу</t>
+          <t>Организация / комиссия</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>Копировальный центр: как заработать не на копейках за копию, а на объёме, если поток — это мелкие разовые заказы у стойки?</t>
+          <t>Свадебное агентство: как выжать максимум из короткого свадебного сезона и не терять комиссию на подрядчиках, срывающих сроки?</t>
         </is>
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>Принимаем файл, правим макет, печатаем и копируем, режем и брошюруем, ламинируем, считаем на кассе и отдаём готовый тираж клиенту.</t>
+          <t>Мы встречаемся с парой, собираем бюджет и концепцию, подбираем площадку и подрядчиков, согласуем тайминг, ведём переписку и предоплаты, а в день свадьбы координируем всех и гасим накладки.</t>
         </is>
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>Копировальный центр: куда уходит прибыль, если очередь за одной копией отвлекает оператора от дорогого широкоформатного тиража?</t>
+          <t>Свадебное агентство: что скрывается за красивой картинкой, если весь год кормит один сезон, а прибыль зависит от чужих подрядчиков?</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>Свадебное агентство: ИИ ведёт рейтинг подрядчиков по истории срывов, срокам и отзывам и подбирает под каждую пару проверенных исполнителей, снижая накладки в день свадьбы и потери комиссии.</t>
         </is>
       </c>
     </row>
@@ -4333,6 +4884,11 @@
           <t>Производитель пластиковых изделий: почему при работающих станках цех в минусе, если долгая переналадка форм и брак литья дороже самой партии?</t>
         </is>
       </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>Производитель пластиковых изделий: ИИ по параметрам ТПА и износу пресс-форм предсказывает сбой и дефект литья, снижая брак партии и внеплановые простои на переналадке.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -4368,6 +4924,11 @@
           <t>SPA-салон: куда утекает выручка, если массаж на полтора часа занимает кабинет и мастера, а гость приходит один раз и не возвращается?</t>
         </is>
       </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>SPA-салон: ИИ по частоте визитов и услугам выявляет уходящих гостей и запускает триггерные предложения абонемента и напоминания, возвращая часть разовых гостей в повторные.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -4395,12 +4956,17 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>Согласуем меню и число гостей, считаем закупку, готовим на производстве, грузим еду и посуду, накрываем на площадке, обслуживаем банкет и убираем.</t>
+          <t>Согласуем меню и число гостей, считаем закупку и порции, нанимаем официантов под заказ, готовим на производстве, грузим еду и посуду, накрываем и обслуживаем банкет на площадке, убираем.</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
         <is>
           <t>Кейтеринговая компания: почему банкет с крупным чеком уходит в ноль, если переготовили порции, а логистика и подменный персонал съели маржу?</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>Кейтеринговая компания: ИИ по числу гостей, меню и истории банкетов прогнозирует порции и нужное число официантов, срезая перепроизводство и списание еды и лишний подменный персонал.</t>
         </is>
       </c>
     </row>
@@ -4438,6 +5004,11 @@
           <t>Зоомагазин: куда уходит прибыль, если покупатель берёт мешок корма раз в месяц, а маркетплейс уже возит тот же корм дешевле?</t>
         </is>
       </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>Зоомагазин: ИИ по весу упаковки и питомцу прогнозирует, когда закончится корм, и шлёт триггерное напоминание с автозаказом, поднимая повторные покупки и удерживая клиента от маркетплейса.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -4473,6 +5044,11 @@
           <t>Производитель бытовой химии: почему объёмы растут, а прибыль стоит, если тара и логистика съедают наценку, а сети платят с отсрочкой?</t>
         </is>
       </c>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>Производитель бытовой химии: ИИ отслеживает цены на сырьё и тару и оптимизирует сроки и объёмы закупок по поставщикам, снижая себестоимость партии и защищая маржу от роста цен.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -4508,6 +5084,11 @@
           <t>Микрофинансовая организация: правда ли, что высокая ставка не спасает, если несколько невозвратов съедают процент, заработанный на сотне добросовестных клиентов?</t>
         </is>
       </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>Микрофинансовая организация: поведенческий скоринг заёмщика по заявке, платёжной истории и альтернативным данным точнее отсеивает невозврат, позволяя наращивать выдачу без роста доли просрочки.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -4535,12 +5116,17 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Выезжаем на участок, готовим проект и смету, завозим растения и грунт, сажаем и монтируем полив, сдаём объект и берём на обслуживание.</t>
+          <t>Выезжаем на участок, готовим проект и смету, ведём земляные работы и дренаж, укладываем дорожки и газон, высаживаем растения, монтируем автополив, берём объект на сезонное обслуживание.</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
           <t>Ландшафтная компания: куда утекает прибыль, если растения не прижились по гарантии, а короткий сезон должен окупить простой всей зимы?</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>Ландшафтная компания: ИИ подбирает растения под свет, почву и климат участка, снижая гибель посадок по гарантии и повторные выезды на пересадку в короткий сезон.</t>
         </is>
       </c>
     </row>
@@ -4570,12 +5156,17 @@
       </c>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>Снимаем бриф, строим стратегию, запускаем кампании, ведём рекламу, готовим отчёты, созваниваемся с клиентом и удерживаем его на следующий месяц.</t>
+          <t>Снимаем бриф и цели, готовим медиаплан по каналам, запускаем контекст и таргет, ведём ставки и креативы, сводим аналитику по лидам и стоимости заявки.</t>
         </is>
       </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
           <t>Digital-маркетинговое агентство: почему при полном портфеле маржа тает, если клиент уходит через три месяца, а на его отчёты ушло больше, чем он заплатил?</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>Digital-маркетинговое агентство: ИИ управляет ставками и распределением бюджета по каналам и креативам, стабилизируя стоимость заявки и ДРР, что удлиняет жизнь клиента на абоненте.</t>
         </is>
       </c>
     </row>
@@ -4613,6 +5204,11 @@
           <t>Карьерный консультант: куда упирается доход, если эксперт продаёт свои часы поштучно, а клиент после первой консультации пропадает?</t>
         </is>
       </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>Карьерный консультант: ИИ-тренажёр на базе методик эксперта разбирает резюме и проводит мок-собеседования между сессиями, превращая разовую консультацию в платное сопровождение до оффера.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -4648,6 +5244,11 @@
           <t>Обувная мастерская: почему при полной приёмке касса маленькая, если мастер тратит время на набойки за копейки вместо дорогой замены подошвы?</t>
         </is>
       </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>Обувная мастерская: ИИ при приёмке по фото износа предлагает выгодные допработы — замену подошвы, профилактику, покраску, — поднимая средний чек вместо копеечных набоек.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -4683,6 +5284,11 @@
           <t>Интернет-магазин автозапчастей: куда утекает прибыль, если из-за одной ошибки в подборе деталь едет назад, а клиент уходит к конкуренту?</t>
         </is>
       </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-магазин автозапчастей: ИИ по VIN подбирает деталь и аналоги с проверкой совместимости, срезая ошибки подбора и дорогие возвраты несовместимых запчастей за счёт магазина.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -4718,6 +5324,11 @@
           <t>Бар: правда ли, что недолив, бесплатные «угощения» друзьям бармена и бой за стойкой утекают мимо кассы быстрее, чем растёт выручка?</t>
         </is>
       </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>Бар: ИИ сверяет пробитые чеки, расход бутылок и весовые остатки, выявляя недолив, бой и бесплатные «угощения» бармена; расхождение по стойке сокращается, а списания под контролем.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -4753,6 +5364,11 @@
           <t>Производитель медицинских расходников: почему завод работает в три смены, а прибыль оседает в неснижаемых остатках склада и партиях с истекающим сроком?</t>
         </is>
       </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>Производитель медицинских расходников: прогноз спроса по истории отгрузок и тендерам планирует размер партий и стерилизацию, снижая неснижаемые остатки и списание партий с истекающим сроком годности.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -4788,6 +5404,11 @@
           <t>Парк аттракционов: куда утекает сезонная касса, если очереди огромные, а половина каруселей в час пик простаивает из-за поломок и нехватки операторов?</t>
         </is>
       </c>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>Парк аттракционов: предиктивное обслуживание по вибрации и телеметрии приводов предсказывает поломки каруселей до часа пик, сокращая внеплановые простои и потерю билетной выручки в очередях.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -4823,6 +5444,11 @@
           <t>Складской оператор: почему склад забит под потолок, а маржа тает, когда половина ячеек занята неликвидом, за который клиент почти не платит?</t>
         </is>
       </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>Складской оператор: ИИ анализирует оборачиваемость груза по ячейкам и предлагает динамический тариф на залежавшийся неликвид, освобождая места под ходовой товар и поднимая доход с квадратного метра.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -4858,6 +5484,11 @@
           <t>Патентное бюро: правда ли, что дороже всего обходятся не сложные заявки, а бесплатные консультации, которые так и не превращаются в договор?</t>
         </is>
       </c>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>Патентное бюро: ИИ-ассистент патентного поиска по базам заявок и публикаций за минуты находит близкие аналоги и черновик формулы, сокращая ручные часы поверенного на каждую заявку.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -4893,6 +5524,11 @@
           <t>Бизнес-коуч: что скрывается за плотным расписанием, если весь доход держится на одном человеке, а после отпуска записи стабильно проседают?</t>
         </is>
       </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>Бизнес-коуч: ИИ-ассистент на методологии коуча ведёт клиентов между сессиями — отвечает на вопросы, напоминает о заданиях, фиксирует прогресс, — масштабируя работу за пределы живых часов.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -4928,6 +5564,11 @@
           <t>Часовая мастерская: куда уходит прибыль, если мастер тратит день на десяток батареек по 300 рублей, а дорогой ремонт механики ждёт неделями?</t>
         </is>
       </c>
+      <c r="H128" s="3" t="inlineStr">
+        <is>
+          <t>Часовая мастерская: по фото часов и механизма ИИ определяет модель и неисправность, сразу оценивает сложный ремонт и апселлит его вместо копеечной батарейки, поднимая средний чек.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -4963,6 +5604,11 @@
           <t>Интернет-магазин товаров для животных: сколько магазин теряет на каждом мешке корма, пока покупатель не добавит в корзину игрушки, лакомства и витамины?</t>
         </is>
       </c>
+      <c r="H129" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-магазин товаров для животных: рекомендации по виду и весу питомца из истории заказов добавляют к мешку корма лакомства, игрушки и витамины, поднимая средний чек и маржу корзины.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -4998,6 +5644,11 @@
           <t>Страховая компания: где утекает прибыль, если полисов продано много, а маржа сгорает на выплатах по недооценённым рискам и мошеннических заявлениях?</t>
         </is>
       </c>
+      <c r="H130" s="3" t="inlineStr">
+        <is>
+          <t>Страховая компания: риск-скоринг по данным заявителя, истории убытков и внешним признакам точнее назначает тариф недооценённым рискам, снижая убыточность портфеля и выплаты по заниженным полисам.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
@@ -5033,6 +5684,11 @@
           <t>SEO-агентство: правда ли, что деньги теряются не на продвижении, а на клиентах, которые уходят за месяц до того, как сайт наконец выстрелил?</t>
         </is>
       </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>SEO-агентство: прогноз оттока по динамике позиций, вовлечённости в отчёты и активности клиента заранее подсвечивает уходящих до результата, запуская удержание и продлевая срок жизни договора.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
@@ -5068,6 +5724,11 @@
           <t>Массажная студия: сколько студия теряет на простоях между сеансами, если руки массажиста заняты, а разовые гости так и не возвращаются на курс?</t>
         </is>
       </c>
+      <c r="H132" s="3" t="inlineStr">
+        <is>
+          <t>Массажная студия: ИИ оптимизирует расписание кабинетов и массажистов, подставляя записи в дыры между сеансами и предлагая ближайшие слоты, поднимая утилизацию кресел и сокращая простои.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
@@ -5103,6 +5764,11 @@
           <t>Квест-комната: почему касса делается за два вечера выходных, а в будни дорогие комнаты стоят пустыми и просто жгут аренду?</t>
         </is>
       </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>Квест-комната: динамическое ценообразование по спросу на слоты делает будни дешевле, а пиковые выходные дороже, выравнивая загрузку комнат и поднимая выручку с простаивающих будних часов.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
@@ -5138,6 +5804,11 @@
           <t>Компания умного дома: что ломается первым, когда проектов много, а прибыль съедают бесконечные доработки сценариев и выезды по гарантии к капризным клиентам?</t>
         </is>
       </c>
+      <c r="H134" s="3" t="inlineStr">
+        <is>
+          <t>Компания умного дома: по параметрам объекта ИИ автоматически собирает спецификацию оборудования, смету и типовые сценарии, снижая зависимость от дефицитных инженеров и ускоряя выпуск коммерческого предложения.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
@@ -5173,6 +5844,11 @@
           <t>Аудиторская фирма: куда уходит маржа, если весь год держится на трёх месяцах отчётности, а дорогие специалисты тонут в ручной сверке документов?</t>
         </is>
       </c>
+      <c r="H135" s="3" t="inlineStr">
+        <is>
+          <t>Аудиторская фирма: ИИ извлекает и сверяет данные из первички — счетов, актов, накладных — с учётными регистрами, снимая с аудиторов ручную сверку и разгружая пик сезона отчётности.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -5208,6 +5884,11 @@
           <t>Производитель электроники: почему при полном цехе заказов прибыль застревает в складе компонентов, которые устаревают раньше, чем уходят в производство?</t>
         </is>
       </c>
+      <c r="H136" s="3" t="inlineStr">
+        <is>
+          <t>Производитель электроники: ИИ оптимизирует закупки компонентов, сопоставляя цены, сроки и надёжность поставщиков и подсказывая аналоги, сокращая замороженные остатки и риск устаревания складских плат.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
@@ -5215,7 +5896,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Паб</t>
+          <t>Кальянная</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -5230,17 +5911,22 @@
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>Паб: как поднять средний чек вечера, если гости берут одно пиво и сидят часами, а кухня почти не работает?</t>
+          <t>Кальянная: как повысить оборот столов и загрузку кальянных мастеров, чтобы вечерний пик не упирался в нехватку рук?</t>
         </is>
       </c>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>Закупаем пиво и продукты, наливаем разливное, готовим закуски, обслуживаем столы и барную стойку, включаем трансляции и списываем остатки в конце смены.</t>
+          <t>Мы встречаем гостей, подбираем табак и чашу под вкус, забиваем и разжигаем кальян, ведём стол весь вечер, меняем угли, пробиваем чек и готовим место под следующую посадку.</t>
         </is>
       </c>
       <c r="G137" s="3" t="inlineStr">
         <is>
-          <t>Паб: почему по вечерам аншлаг, а маржу тихо выпивают недолив, бой посуды и бочки, которые выдыхаются раньше, чем их допьют?</t>
+          <t>Кальянная: почему зал полон, а касса пустеет, если один стол занят до полуночи под один кальян и чайник чая?</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="inlineStr">
+        <is>
+          <t>Кальянная: прогноз вечерней нагрузки по истории посадок и дню недели планирует смены кальянных мастеров, чтобы в пик хватало рук, ускоряя оборот столов без переплаты в тихие часы.</t>
         </is>
       </c>
     </row>
@@ -5278,6 +5964,11 @@
           <t>Страховой брокер: правда ли, что вся прибыль в пролонгациях, а брокер каждый год заново гоняется за клиентом, забывая напомнить о продлении?</t>
         </is>
       </c>
+      <c r="H138" s="3" t="inlineStr">
+        <is>
+          <t>Страховой брокер: ИИ отслеживает даты окончания полисов и заранее запускает триггерные напоминания о пролонгации с готовым сравнением предложений, повышая долю продлений и возвращая ускользающую комиссию.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
@@ -5313,6 +6004,11 @@
           <t>Интернет-магазин цветов и подарков: почему в праздники срываются доставки ко времени, а в будни свежий букет вянет на складе быстрее, чем поступит заказ?</t>
         </is>
       </c>
+      <c r="H139" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-магазин цветов и подарков: ИИ планирует маршруты и временные окна курьеров под праздничный пик, снижая срывы доставки ко времени и число опозданий по заказам на конкретный час.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
@@ -5348,6 +6044,11 @@
           <t>Мувинговая компания: куда уходит прибыль, если машина в разъездах весь день, а платят лишь за пару часов погрузки, пока грузчики стоят в пробках?</t>
         </is>
       </c>
+      <c r="H140" s="3" t="inlineStr">
+        <is>
+          <t>Мувинговая компания: ИИ оптимизирует маршруты и стыкует заказы бригад по районам и объёму, сокращая простои грузчиков между переездами и холостые пробеги, поднимая маржу с машины за день.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
@@ -5375,12 +6076,17 @@
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>Заказываем книги у издательств, расставляем по разделам, консультируем покупателей, продаём через кассу, возвращаем нераспроданное и проводим встречи с авторами.</t>
+          <t>Заказываем книги у издательств, расставляем по разделам, консультируем и продаём на кассе, предлагаем сопутку и кофе, возвращаем нераспроданные тиражи издателю и проводим встречи с авторами.</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
           <t>Книжный магазин: правда ли, что деньги делает не книга, а кофе, канцелярия и сувениры, пока бестселлеры лишь заманивают людей внутрь?</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="inlineStr">
+        <is>
+          <t>Книжный магазин: ИИ анализирует продажи по разделам и оборачиваемость полок, помечая неходовые тиражи к возврату издателю и высвобождая квадратные метры под кофе, канцелярию и ходовые новинки.</t>
         </is>
       </c>
     </row>
@@ -5418,6 +6124,11 @@
           <t>Веб-студия: выглядит прибыльным проект с согласованной сметой, но почему разработчики месяцами доделывают правки, которые клиент считает мелочью?</t>
         </is>
       </c>
+      <c r="H142" s="3" t="inlineStr">
+        <is>
+          <t>Веб-студия: ИИ генерирует вёрстку типовых блоков, тексты и обработку фото по брендбуку, сокращая нормо-часы на бесконечные правки и защищая заложенную маржу проектов с фиксированной ценой.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -5453,6 +6164,11 @@
           <t>Налоговый консалтинг: что скрывается за высоким чеком, если самые ценные советы звучат на бесплатной встрече, а платит клиент, только когда прижмёт проверка?</t>
         </is>
       </c>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>Налоговый консалтинг: скоринг входящих заявок по отрасли, оборотам и признакам налоговых рисков приоритизирует бесплатные встречи, доводя до платного договора реально конвертируемых клиентов и экономя часы экспертов.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
@@ -5488,6 +6204,11 @@
           <t>Производитель светильников: можно ли расти, если портфель заказов полон, а деньги заморожены в остатках моделей, вышедших из моды раньше продажи?</t>
         </is>
       </c>
+      <c r="H144" s="3" t="inlineStr">
+        <is>
+          <t>Производитель светильников: прогноз спроса по моделям с учётом сезона и трендов планирует производство и закупку комплектующих, сокращая заморозку денег в остатках вышедших из моды позиций.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
@@ -5523,6 +6244,11 @@
           <t>Управляющая компания коммерческой недвижимости: куда утекает прибыль, если здание заполнено, а маржу съедают простой между арендаторами, долги и авральный ремонт систем?</t>
         </is>
       </c>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>Управляющая компания коммерческой недвижимости: предиктивное обслуживание инженерных систем по телеметрии и истории заявок предупреждает аварии до отказа, снижая авральные ремонты и простои площадей между арендаторами.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
@@ -5550,12 +6276,17 @@
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>Строим стратегию, пишем пресс-релизы, налаживаем связи с журналистами, размещаем публикации, ведём соцсети клиента и отчитываемся об охватах и упоминаниях.</t>
+          <t>Строим PR-стратегию, готовим инфоповоды и пресс-релизы, питчим темы журналистам, согласуем и размещаем публикации, мониторим упоминания и тональность, сводим отчёт об охватах.</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
           <t>PR-агентство: правда ли, что клиент уходит не из-за плохой работы, а потому что не видит в отчёте цифру, которую можно связать с продажами?</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>PR-агентство: ИИ мониторит упоминания бренда, считает тональность и долю голоса из публикаций и соцсетей, превращая размытую работу в цифры отчёта и удерживая клиента на абонплате.</t>
         </is>
       </c>
     </row>
@@ -5585,12 +6316,17 @@
       </c>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>Привлекаем трафик, продаём курс через вебинар, зачисляем ученика, ведём по урокам, проверяем домашки силами кураторов и выдаём сертификат.</t>
+          <t>Привлекаем трафик, продаём курс через вебинар, зачисляем ученика, ведём по урокам с поддержкой кураторов, проверяем домашки и защиту проектов, доводим до результата и помогаем с трудоустройством.</t>
         </is>
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
           <t>Онлайн-школа профессиональных навыков: куда утекают деньги на рекламу, если купивших много, а курс до конца проходит горстка, и рекомендаций почти нет?</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>Онлайн-школа профессиональных навыков: прогноз оттока по активности в уроках и сдаче домашек заранее выявляет уходящих учеников, запуская интервенции кураторов и повышая долю дошедших до финала.</t>
         </is>
       </c>
     </row>
@@ -5628,6 +6364,11 @@
           <t>Цветочный магазин: почему 8 марта не хватает ни рук, ни товара, а в обычную неделю половина роз с витрины уезжает в мусорный бак?</t>
         </is>
       </c>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>Цветочный магазин: прогноз списаний по срокам жизни цветка и спросу оптимизирует ежедневную закупку на базе, сокращая долю увядшего в мусор между праздниками без дефицита в пиковые дни.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
@@ -5663,6 +6404,11 @@
           <t>Таксопарк: куда утекает прибыль, если машины на линии круглосуточно, а маржу выедают авто без водителей, ремонты и вечная текучка за рулём?</t>
         </is>
       </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>Таксопарк: ИИ подбирает и скринит водителей под простаивающие машины и распределяет смены по спросу, сокращая долю авто без водителей и текучку, поднимая выручку с каждой машины.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
@@ -5698,6 +6444,11 @@
           <t>Боулинг-клуб: правда ли, что дорожки едва отбивают аренду, а прибыль приносят бар и кухня, пока сломанный пинсеттер режет выходную кассу?</t>
         </is>
       </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>Боулинг-клуб: динамическое ценообразование по загрузке дорожек и дню недели наполняет пустые будни выгодными пакетами игры с баром, поднимая выручку с дорожки без потери выходной маржи.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
@@ -5733,6 +6484,11 @@
           <t>Тату-студия: что скрывается за очередью к топовому мастеру, если студия зарабатывает на аренде кресла, а вся база клиентов принадлежит не ей?</t>
         </is>
       </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>Тату-студия: ИИ примеряет эскиз на фото тела клиента в нужном месте и размере, повышая конверсию консультаций в предоплату и делая воронку эскизов активом студии, а не мастера.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
@@ -5760,12 +6516,17 @@
       </c>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>Принимаем залог, выдаём инструмент по договору, инструктируем по использованию, принимаем назад, проверяем и обслуживаем, ремонтируем и списываем изношенное.</t>
+          <t>Проверяем документы, берём залог и оплату за срок, выдаём исправный инструмент с инструктажем, принимаем назад, оцениваем износ, удерживаем за поломки из залога, обслуживаем и списываем изношенное.</t>
         </is>
       </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
           <t>Пункт проката инструмента: почему самый дорогой перфоратор простаивает и не окупается, а ходовую технику клиенты возвращают убитой?</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>Пункт проката инструмента: предиктивное ТО по наработке моточасов и истории аренд каждой позиции — планово меняем расходники до поломки, сокращаем аварийный простой парка и растим доход с единицы.</t>
         </is>
       </c>
     </row>
@@ -5803,6 +6564,11 @@
           <t>Производитель ювелирных изделий: почему при растущей цене золота склад дорожает, а прибыль тает, если ходовые артикулы вечно в дефиците, а неликвид висит витриной?</t>
         </is>
       </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>Производитель ювелирных изделий: прогноз спроса по артикулам, пробам и размерам на истории продаж и сезонности — держим ходовое в наличии, режем неликвид на складе и высвобождаем замороженную в остатках оборотку.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
@@ -5838,6 +6604,11 @@
           <t>Дизайн-студия: куда утекает прибыль проекта, когда пятый круг бесплатных правок и вечное «сделайте повеселее» превращают фикс-бюджет в работу себе в убыток?</t>
         </is>
       </c>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>Дизайн-студия: генеративный ИИ по брифу и референсам выдаёт 3–5 концепций за час — заказчик выбирает направление на старте, круги правок сокращаются, а фикс-бюджет перестаёт уходить в убыток.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
@@ -5873,6 +6644,11 @@
           <t>Коворкинг: почему при полной продаже мест зал полупустой, а переговорки то простаивают, то не забронировать, если резиденты платят за воздух, которым не пользуются?</t>
         </is>
       </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>Коворкинг: компьютерное зрение считает реальную загрузку столов и переговорных по камерам — видим, что фикс-места пустуют, переводим их в гибкий тариф и продаём одно место дважды, поднимая доход с метра.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -5908,6 +6684,11 @@
           <t>Студия мобильных приложений: правда ли, что прибыль сгорает не в разработке, а в недооценённых спринтах и доработках, которые заказчик считает «мелкими правками»?</t>
         </is>
       </c>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>Студия мобильных приложений: ИИ оценивает спринты по истории похожих задач и трудозатрат в трекере — точнее считаем смету, закладываем поддержку релизов в бюджет и перестаём работать в минус на недооценке.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
@@ -5935,12 +6716,17 @@
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заявки, распределяем машины и водителей, встречаем у прилёта, везём по маршруту, отслеживаем задержки рейсов и закрываем поездки в отчётность.</t>
+          <t>Принимаем заявки, распределяем машины и водителей, отслеживаем табло и задержки рейсов, корректируем время подачи, встречаем у прилёта, везём по маршруту и закрываем поездки в отчётность.</t>
         </is>
       </c>
       <c r="G157" s="3" t="inlineStr">
         <is>
           <t>Трансферная компания: сколько прибыли уезжает порожняком, когда водитель час ждёт задержанный рейс, а обратно из аэропорта едет с пустым салоном?</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>Трансферная компания: ИИ строит маршруты и сцепляет подачи с обратными рейсами по табло прилётов и заявкам — меньше порожнего пробега и ожидания у прилёта, выше загрузка машины и маржа рейса.</t>
         </is>
       </c>
     </row>
@@ -5978,6 +6764,11 @@
           <t>Груминг-салон: куда утекает выручка, когда клиент срывается в день визита, мастер простаивает между записями, а «просто помыть» занимает столько же кресла, сколько сложная стрижка?</t>
         </is>
       </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>Груминг-салон: ИИ-расписание подбирает слот под длительность услуги и уплотняет окна между стрижками, прогнозируя срывы записи — простой кресел падает, мастер загружен ровно, выручка с кресла растёт.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n">
@@ -6013,6 +6804,11 @@
           <t>Тендерное агентство: почему специалист тонет в сотнях закупок вручную, пропуская тендер с идеальным лотом, пока разбирает те, где клиент заведомо не проходит?</t>
         </is>
       </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>Тендерное агентство: ИИ отбирает из тысяч закупок только подходящие профилю и допускам клиента, ранжируя по шансу победы — специалист не тонет в ручном разборе и не пропускает идеальный лот.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
@@ -6020,7 +6816,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Бильярдный клуб</t>
+          <t>Компьютерный клуб (киберарена)</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -6035,17 +6831,22 @@
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>Бильярдный клуб: как поднять выручку со стола в час и загрузку днём, если касса делается только вечером и в выходные?</t>
+          <t>Компьютерный клуб (киберарена): как поднять почасовую загрузку в будни и отбить апгрейд железа, пока оно не устарело?</t>
         </is>
       </c>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>Сдаём столы по часам, выдаём кии и шары, ведём учёт времени игры, продаём бар и кухню, обслуживаем турниры и закрываем счёт по партии.</t>
+          <t>Мы сажаем гостей за станции, продаём часы и абонементы, следим за турнирами и бронями, подкручиваем настройки и обновляем игры, чистим и апгрейдим железо, докручиваем выручку баром и снеками.</t>
         </is>
       </c>
       <c r="G160" s="3" t="inlineStr">
         <is>
-          <t>Бильярдный клуб: выглядит прибыльно вечером, но куда девается маржа, если днём столы пустуют, а весь бар держится на пиве по пятницам?</t>
+          <t>Компьютерный клуб (киберарена): что съедает маржу, если днём залы пустуют, а вечерний аншлаг не отбивает новые видеокарты?</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="inlineStr">
+        <is>
+          <t>Компьютерный клуб (киберарена): динамические тарифы по часам и дням недели на истории загрузки станций поднимают дневную и будничную посадку и ускоряют окупаемость апгрейда железа.</t>
         </is>
       </c>
     </row>
@@ -6083,6 +6884,11 @@
           <t>Ювелирный магазин: сколько денег заморожено в витрине, если ходовые размеры вечно кончаются перед 8 марта, а неликвид годами блестит под стеклом?</t>
         </is>
       </c>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>Ювелирный магазин: ИИ-рекомендации подбирают украшение под повод, бюджет и прошлые покупки клиента и предлагают комплект — растёт средний чек и конверсия консультации без дополнительного трафика.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n">
@@ -6118,6 +6924,11 @@
           <t>Столовая: почему при полной очереди в обед прибыль тает, если к вечеру половина линии раздачи уезжает в списание, а завтрашнее меню приходится угадывать заново?</t>
         </is>
       </c>
+      <c r="H162" s="3" t="inlineStr">
+        <is>
+          <t>Столовая: ИИ прогнозирует спрос по блюдам на день с учётом дня недели и погоды и подсказывает объём готовки — меньше списаний вечерней раздачи, точнее закупка, меню не приходится угадывать.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n">
@@ -6145,12 +6956,17 @@
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>Закупаем пряжу и сырьё, ткём и красим полотно, кроим и шьём партии, проверяем качество, комплектуем заказы и отгружаем оптовикам и швейным цехам.</t>
+          <t>Закупаем пряжу, ткём или вяжем полотно, красим и отделываем, проверяем плотность и цвет, режем в рулоны, комплектуем заказы и отгружаем швейным фабрикам и оптовикам.</t>
         </is>
       </c>
       <c r="G163" s="3" t="inlineStr">
         <is>
           <t>Производитель текстиля: куда уходит прибыль, когда станки то простаивают в межсезонье, то не успевают в пик, а рулоны непроданного полотна пылятся на складе?</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>Производитель текстиля: прогноз заказов по сезонности и истории клиентов планирует загрузку станков и объём полотна — меньше простоя в межсезонье и авралов в пик, склад перестаёт лежать мёртвым капиталом.</t>
         </is>
       </c>
     </row>
@@ -6188,6 +7004,11 @@
           <t>Интернет-магазин продуктов: правда ли, что на каждом заказе теряешь, если скоропорт летит в списание, курьер везёт три пакета, а покупатель отменяет на пороге?</t>
         </is>
       </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-магазин продуктов: ИИ управляет заказом скоропорта и уценкой по срокам годности и скорости продаж — режем списания, распродаём близкие к сроку позиции вовремя и удерживаем маржу на заказе.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
@@ -6215,12 +7036,17 @@
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Собираем документы клиента, оцениваем платёжеспособность, подаём заявки в банки, подбираем программу, сопровождаем одобрение и доводим до сделки у нотариуса.</t>
+          <t>Собираем документы клиента, оцениваем платёжеспособность, подбираем программу, подаём заявки в несколько банков, добиваемся одобрения и сопровождаем клиента до подписания кредитного договора и регистрации сделки.</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
           <t>Ипотечный брокер: куда утекает комиссия, если клиент неделями собирает справки, банк отказывает на финише, а до сделки доходит один из пяти?</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="inlineStr">
+        <is>
+          <t>Ипотечный брокер: скоринг заявки по доходу, кредитной истории и требованиям банков предсказывает вероятность одобрения — подаём клиента только туда, где одобрят, растёт доля сделок и комиссия, меньше пустых подач.</t>
         </is>
       </c>
     </row>
@@ -6250,12 +7076,17 @@
       </c>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>Привлекаем через пробный урок, распределяем по группам и педагогам, ведём занятия на платформе, проверяем домашки, отслеживаем прогресс и продлеваем абонемент.</t>
+          <t>Привлекаем через пробный урок, распределяем детей по группам и педагогам, ведём занятия на платформе, проверяем домашки, отслеживаем прогресс, регулярно показываем результат родителям и продлеваем абонемент.</t>
         </is>
       </c>
       <c r="G166" s="3" t="inlineStr">
         <is>
           <t>Онлайн-школа для детей: почему деньги на привлечение сгорают, если ребёнок бросает после пробного, родитель не видит прогресса, а до конца курса доходит меньше половины?</t>
+        </is>
+      </c>
+      <c r="H166" s="3" t="inlineStr">
+        <is>
+          <t>Онлайн-школа для детей: ИИ по активности на платформе, посещаемости и проверке домашек предсказывает риск бросить после пробного — триггерные касания и отчёт родителю удерживают ученика до конца курса, растёт LTV.</t>
         </is>
       </c>
     </row>
@@ -6285,12 +7116,17 @@
       </c>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>Обследуем процессы заказчика, проектируем архитектуру, внедряем и настраиваем системы, интегрируем их между собой, обучаем пользователей и берём на сопровождение.</t>
+          <t>Обследуем процессы заказчика, проектируем архитектуру, внедряем и настраиваем системы, переносим данные и интегрируем их между собой, обучаем пользователей и берём на сопровождение.</t>
         </is>
       </c>
       <c r="G167" s="3" t="inlineStr">
         <is>
           <t>IT-консалтинг и системная интеграция: где растворяется прибыль проекта, когда сроки внедрения плывут, дорогие специалисты латают старые интеграции, а заказчик считает это гарантией?</t>
+        </is>
+      </c>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>IT-консалтинг и системная интеграция: RAG-ассистент по документации проектов и регламентам отвечает на типовые вопросы поддержки — первая линия закрывает обращения без сеньоров, дорогие специалисты возвращаются к внедрениям.</t>
         </is>
       </c>
     </row>
@@ -6328,6 +7164,11 @@
           <t>Караоке-клуб: выглядит золотой жилой по выходным, но куда уходит прибыль, если в будни кабинки пустуют, а весь чек держится на баре в две ночи?</t>
         </is>
       </c>
+      <c r="H168" s="3" t="inlineStr">
+        <is>
+          <t>Караоке-клуб: динамическое ценообразование на будни и дневные часы по истории броней — заполняем пустые кабинки в непиковое время скидкой и депозитом, поднимаем выручку с зала и загрузку будней.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
@@ -6363,6 +7204,11 @@
           <t>Служба дезинсекции: почему прибыль зависит от погоды, если летом бригады не справляются, зимой простаивают, а клиент вызывает, лишь когда «уже совсем достали»?</t>
         </is>
       </c>
+      <c r="H169" s="3" t="inlineStr">
+        <is>
+          <t>Служба дезинсекции: ИИ прогнозирует поток заявок по сезону, погоде и району и планирует смены бригад — нет простоя зимой и срывов в летний пик, выше загрузка выездов и повторные обработки в графике.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
@@ -6398,6 +7244,11 @@
           <t>Мини-склады self-storage: сколько дохода стоят пустые боксы, если арендатор занимает ячейку на месяц, съезжает без предупреждения, а должники годами держат замок?</t>
         </is>
       </c>
+      <c r="H170" s="3" t="inlineStr">
+        <is>
+          <t>Мини-склады self-storage: ИИ по платёжному поведению и сроку аренды предсказывает, кто съедет или уйдёт в просрочку — триггерные удержания и своевременная работа с должниками поднимают заполняемость и доход с метра.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
@@ -6425,12 +7276,17 @@
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>Закупаем и брендируем парк, распределяем машины по районам, пускаем клиентов через приложение, чистим и заправляем авто, чиним поломки и штрафуем за нарушения.</t>
+          <t>Закупаем и брендируем парк, верифицируем водителей в приложении, распределяем и релоцируем машины под спрос по районам, чистим и заправляем авто, обслуживаем поломки и штрафуем за нарушения.</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
         <is>
           <t>Каршеринг: куда утекает прибыль с машины, если утром весь парк на окраине, вечером его не найти в центре, а один лихач в ремонте съедает выручку десяти поездок?</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>Каршеринг: ИИ прогнозирует спрос по районам и часам и планирует релокацию машин с окраин в центр — меньше простоя авто, выше число поездок и доход с машины в сутки.</t>
         </is>
       </c>
     </row>
@@ -6468,6 +7324,11 @@
           <t>Фудтрак: почему хорошая точка не гарантирует прибыль, если дождь обнуляет день, очередь стоит один час, а заготовки к вечеру летят в мусор?</t>
         </is>
       </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>Фудтрак: прогноз продаж по локации, погоде и дню недели на истории точек задаёт объём заготовок на смену — меньше порчи к вечеру и упущенных продаж в час пик, стабильнее маржа точки.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
@@ -6503,6 +7364,11 @@
           <t>Онлайн-аптека: где теряется прибыль, если наценку на жизненно важные лекарства ограничили сверху, а редкие препараты списываются по сроку годности непроданными?</t>
         </is>
       </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>Онлайн-аптека: ИИ-рекомендации предлагают к рецептурному заказу сопутствующие безрецептурные товары и БАДы по корзине и истории — при зарегулированной наценке растёт средний чек и маржа заказа.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
@@ -6538,6 +7404,11 @@
           <t>Производитель снеков: куда девается маржа пачки, если сеть требует ретробонус, полка держится на бесконечных акциях, а линия то стоит, то работает в три смены?</t>
         </is>
       </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>Производитель снеков: ИИ считает эффективность промо по сетям и SKU и распределяет трейд-бюджет на работающие акции — режем бесполезные скидки и ретробонусы, удерживаем маржу пачки на полке.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
@@ -6573,6 +7444,11 @@
           <t>Сертификационный центр: почему оформление тянется неделями, если эксперт вручную сверяет каждый документ, а заявка гуляет между клиентом и лабораторией по десять раз?</t>
         </is>
       </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>Сертификационный центр: ИИ извлекает и сверяет данные из документов заявителя с требованиями и протоколами лаборатории — уходит ручная проверка эксперта, оформление ускоряется с недель до дней, растёт пропускная способность.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
@@ -6608,6 +7484,11 @@
           <t>UX/UI-студия: правда ли, что прибыль проекта убивают не сложные экраны, а бесконечные «давайте передвинем кнопку» и правки, которые заказчик не считает работой?</t>
         </is>
       </c>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>UX/UI-студия: ИИ транскрибирует и резюмирует интервью и юзабилити-тесты, вытаскивая инсайты и цитаты — исследование перестаёт быть чёрной дырой по срокам, сеньоры экономят часы на разборе записей.</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
@@ -6643,6 +7524,11 @@
           <t>Фитнес-клуб: почему проданная в январе карта — это убыток, если человек приходит трижды, забрасывает к марту и не продлевается, а на его место продали ещё пять?</t>
         </is>
       </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>Фитнес-клуб: ИИ по частоте посещений и активности после покупки карты предсказывает отток к весне — персональные напоминания и предложения возвращают клиента в зал, растут продления и LTV абонемента.</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
@@ -6670,12 +7556,17 @@
       </c>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>Проводим вводное тестирование, подбираем преподавателя, составляем расписание, ведём занятия, отслеживаем прогресс к экзамену и продлеваем пакет часов.</t>
+          <t>Проводим вводное тестирование, подбираем преподавателя, составляем расписание, ведём занятия, делаем промежуточные срезы и показываем родителям рост баллов, готовим к экзамену и продлеваем пакет часов.</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
         <is>
           <t>Репетиторский центр: куда утекает выручка, если ученик бросает после трёх занятий, родитель не видит роста баллов, а расписание преподавателя дырявое между уроками?</t>
+        </is>
+      </c>
+      <c r="H178" s="3" t="inlineStr">
+        <is>
+          <t>Репетиторский центр: ИИ-расписание уплотняет окна между уроками и подбирает слоты под преподавателя и ученика — простой в расписании падает, загрузка педагогов растёт, освобождается время под новые пакеты часов.</t>
         </is>
       </c>
     </row>
@@ -6705,12 +7596,17 @@
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>Осматриваем вещь, оцениваем объём работ, разбираем и зачищаем, восстанавливаем каркас, перетягиваем и покрываем, собираем и отдаём клиенту.</t>
+          <t>Осматриваем вещь, даём предварительную оценку, разбираем и зачищаем, уточняем смету и сроки по вскрытому объёму, восстанавливаем каркас, перетягиваем и покрываем, собираем и отдаём клиенту.</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
           <t>Студия реставрации мебели: почему смета вечно врёт, если реальный объём работ вскрывается только когда сняли обивку, а клиент уже согласовал старую цену?</t>
+        </is>
+      </c>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>Студия реставрации мебели: ИИ по фото вещи пред-оценивает объём работ и типовые дефекты до разборки — смета точнее с первого осмотра, меньше сюрпризов после вскрытия обивки и споров о цене.</t>
         </is>
       </c>
     </row>
@@ -6748,6 +7644,11 @@
           <t>Магазин спортивных товаров: сколько денег заморожено в остатках, если ходовой размер кроссовок кончается за неделю, а зимняя коллекция висит до мартовской уценки в минус?</t>
         </is>
       </c>
+      <c r="H180" s="3" t="inlineStr">
+        <is>
+          <t>Магазин спортивных товаров: ИИ управляет уценкой несезонных остатков по скорости продаж и остатку сезона — распродаём коллекции до мартовской минусовой уценки, высвобождаем полку и оборотку, держим маржу.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
@@ -6783,6 +7684,11 @@
           <t>Кредитный брокер: куда уходит время впустую, если из десяти клиентов одобряют двоих, банк режет на финише, а неплатёжеспособных видно только после часа переписки?</t>
         </is>
       </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>Кредитный брокер: скоринг по кредитной истории и профилю отсеивает заведомо неплатёжеспособных и подбирает банк с высоким шансом одобрения — специалист не тратит часы впустую, растёт доля выдач и комиссия.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
@@ -6818,6 +7724,11 @@
           <t>Производитель напитков: почему на каждой бутылке зарабатываешь копейки, если сеть требует промо, тяжёлый груз дорого везти, а линия розлива простаивает между заказами?</t>
         </is>
       </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>Производитель напитков: ИИ строит маршруты доставки тяжёлого груза по заказам сетей и дистрибьюторов, объединяя рейсы и снижая пробег и стоимость логистики на бутылку на 15-20%.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n">
@@ -6845,12 +7756,17 @@
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>Собираем бриф клиента, подбираем блогеров под аудиторию, согласуем ТЗ и цену размещения, контролируем выход интеграции, снимаем охваты и вовлечённость, готовим отчёт.</t>
+          <t>Снимаем бриф, подбираем блогеров и проверяем их аудиторию на накрутку, согласуем ТЗ и цену, контролируем выход интеграции, собираем охваты и вовлечённость, готовим отчёт.</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
           <t>Агентство influencer-маркетинга: почему клиент платит за миллионные охваты, а продаж нет — и как отличить живую аудиторию блогера от накрученной ещё до подписания?</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>Агентство influencer-маркетинга: ИИ анализирует динамику подписчиков, комментариев и охватов блогера, выявляя накрутку и ботов до подписания и повышая долю кампаний с реальными продажами.</t>
         </is>
       </c>
     </row>
@@ -6880,12 +7796,17 @@
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>Бронируем столы с депозитом, пускаем гостей через фейс-контроль и гардероб, ставим программу диджеев, продаём бар и кальяны, закрываем счета к утру.</t>
+          <t>Собираем программу диджеев и афишу, бронируем столы с депозитом, пускаем гостей через фейс-контроль и гардероб, продаём бар и кальяны, держим танцпол и закрываем счета к утру.</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
           <t>Ночной клуб: зал забит под завязку, а касса тонкая — куда утекает прибыль, если люди пришли на диджея, но почти ничего не берут в баре?</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="inlineStr">
+        <is>
+          <t>Ночной клуб: ИИ по чекам и профилю гостя за столом подсказывает бармену персональные допродажи бара и кальянов, поднимая средний чек и выручку в будни.</t>
         </is>
       </c>
     </row>
@@ -6923,6 +7844,11 @@
           <t>Прокат автомобилей: половина парка стоит на приколе, а платежи по лизингу идут — сколько прибыли машина съедает за каждый день без клиента?</t>
         </is>
       </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>Прокат автомобилей: ИИ по истории броней прогнозирует спрос по классам и датам и оптимально распределяет парк, сокращая простой машин и покрывая лизинговые платежи загрузкой.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
@@ -6958,6 +7884,11 @@
           <t>Отель: номера заполнены под 90%, а прибыли нет — правда ли, что комиссии агрегаторов и демпинг по тарифу съедают всё, что даёт загрузка?</t>
         </is>
       </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>Отель: ИИ ежедневно пересчитывает тариф по датам, загрузке, спросу и ценам конкурентов, снижая зависимость от скидок агрегаторов и поднимая ADR и доход на номер (RevPAR).</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n">
@@ -6993,6 +7924,11 @@
           <t>Зоогостиница: в праздники мест нет и очередь, а в будни вольеры пустуют — сколько теряет бизнес на том, что спрос приходит всего пару раз в году?</t>
         </is>
       </c>
+      <c r="H187" s="3" t="inlineStr">
+        <is>
+          <t>Зоогостиница: ИИ на данных прошлых броней задаёт динамические цены — скидки в будни и межсезонье, наценку в праздники, — выравнивая загрузку вольеров и повышая заполняемость в низкий сезон.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n">
@@ -7028,6 +7964,11 @@
           <t>Онлайн-магазин одежды: заказов много, а прибыль тает — куда она уходит, если каждый второй клиент заказывает три размера, чтобы вернуть два?</t>
         </is>
       </c>
+      <c r="H188" s="3" t="inlineStr">
+        <is>
+          <t>Онлайн-магазин одежды: ИИ по параметрам покупателя и реальным меркам вещей рекомендует точный размер, снижая заказы «на примерку» и долю возвратов, сохраняя маржу с посылки.</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n">
@@ -7063,6 +8004,11 @@
           <t>Фермерское хозяйство: урожай отличный, а денег мало — почему основную маржу забирают перекупщики, пока часть продукции гниёт на складе?</t>
         </is>
       </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
+          <t>Фермерское хозяйство: ИИ подбирает под каждую партию прямых покупателей — рестораны, сети, опт — по объёму, цене и срокам, снижая долю перекупщиков и поднимая цену реализации.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n">
@@ -7098,6 +8044,11 @@
           <t>Инвестиционная компания: активов под управлением всё больше, а прибыль не растёт — правда ли, что ручная аналитика и отчёты держат бизнес заложником числа сотрудников?</t>
         </is>
       </c>
+      <c r="H190" s="3" t="inlineStr">
+        <is>
+          <t>Инвестиционная компания: ИИ генерирует персональные отчёты по портфелям и рыночные комментарии клиентам из данных, освобождая аналитиков от рутины и позволяя растить активы под управлением без найма.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n">
@@ -7133,6 +8084,11 @@
           <t>Переводческое агентство: заказов поток, а маржа тонкая — сколько времени и денег уходит на ручной подбор исполнителя и вычитку разнобоя в терминах?</t>
         </is>
       </c>
+      <c r="H191" s="3" t="inlineStr">
+        <is>
+          <t>Переводческое агентство: ИИ делает черновой машинный перевод и сверяет термины по глоссарию клиента, оставляя человеку редактуру и ускоряя срочные заказы без потери качества.</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n">
@@ -7168,6 +8124,11 @@
           <t>Магазин детских товаров: полки полные, а деньги заморожены — куда утекает прибыль, если размер 74 не продали, а ребёнок уже носит 86?</t>
         </is>
       </c>
+      <c r="H192" s="3" t="inlineStr">
+        <is>
+          <t>Магазин детских товаров: ИИ прогнозирует спрос по возрастам, размерам и сезонам и планирует закупки, сокращая неликвид и замороженные в остатках деньги на непроданных размерах.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n">
@@ -7203,6 +8164,11 @@
           <t>IT-аутсорсинг для бизнеса: клиентов на абонентке всё больше, а инженеры выгорают — почему фиксированная плата превращается в бесконечный поток мелких заявок?</t>
         </is>
       </c>
+      <c r="H193" s="3" t="inlineStr">
+        <is>
+          <t>IT-аутсорсинг для бизнеса: ИИ-ассистент на базе прошлых тикетов и регламентов сортирует заявки и подсказывает инженерам готовые решения, сокращая время на типовые инциденты при фиксированной абонентке.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
@@ -7238,6 +8204,11 @@
           <t>Частная школа: набор прошёл, классы полные, а к весне парты пустеют — сколько теряет школа на каждом ученике, который ушёл, не доучившись год?</t>
         </is>
       </c>
+      <c r="H194" s="3" t="inlineStr">
+        <is>
+          <t>Частная школа: ИИ по посещаемости, оценкам и оплатам выявляет учеников с риском ухода к середине года и запускает адресную работу с родителями, повышая удержание до конца курса.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n">
@@ -7265,12 +8236,17 @@
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>Обсуждаем проект с клиентом, считаем смету, производим модули на площадке, везём на участок, монтируем и подключаем коммуникации, сдаём готовый дом.</t>
+          <t>Обсуждаем проект, считаем смету и заключаем договор, производим модули в заводском цеху, готовим фундамент на участке, привозим и монтируем блоки, подключаем коммуникации, сдаём дом.</t>
         </is>
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
           <t>Компания модульных домов: заказы есть, а прибыль скачет — почему между сделками цех простаивает, пока клиент месяцами думает и согласует проект?</t>
+        </is>
+      </c>
+      <c r="H195" s="3" t="inlineStr">
+        <is>
+          <t>Компания модульных домов: ИИ по параметрам проекта автоматически считает смету и готовит договор и КП, сокращая срок согласования сделки и простой цеха между заказами.</t>
         </is>
       </c>
     </row>
@@ -7308,6 +8284,11 @@
           <t>Студия персональных тренировок: расписание вроде плотное, а тренер увольняется и уводит клиентов за собой — сколько бизнес теряет на привязке людей к одному человеку?</t>
         </is>
       </c>
+      <c r="H196" s="3" t="inlineStr">
+        <is>
+          <t>Студия персональных тренировок: ИИ подбирает клиенту свободного тренера под цель и график и закрывает окна в расписании, снижая зависимость от одного специалиста и потерю клиентов при увольнении.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
@@ -7343,6 +8324,11 @@
           <t>Тепличное хозяйство: зелень и овощи растут круглый год, а прибыль зависит от счёта за свет — сколько маржи сгорает на отоплении и досветке в морозы?</t>
         </is>
       </c>
+      <c r="H197" s="3" t="inlineStr">
+        <is>
+          <t>Тепличное хозяйство: ИИ прогнозирует выход урожая и оптовую цену и планирует режим досветки и отопления так, чтобы энергозатраты окупались, поднимая рентабельность зимних партий.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
@@ -7378,6 +8364,11 @@
           <t>Детейлинг-центр: запись плотная, мастера в мыле, а касса не радует — почему один бокс на весь день ради одной машины ограничивает весь заработок?</t>
         </is>
       </c>
+      <c r="H198" s="3" t="inlineStr">
+        <is>
+          <t>Детейлинг-центр: ИИ по состоянию авто и истории клиента предлагает выгодные допуслуги — керамику, плёнку, защиту салона, — поднимая средний чек с одного бокса без роста числа постов.</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
@@ -7413,6 +8404,11 @@
           <t>Агентство продвижения на маркетплейсах: продажи клиента растут, а ваша абонентка стоит на месте — куда девается маржа, когда каждую карточку и ставку крутят руками?</t>
         </is>
       </c>
+      <c r="H199" s="3" t="inlineStr">
+        <is>
+          <t>Агентство продвижения на маркетплейсах: ИИ управляет ставками и бюджетом рекламы по каждой карточке, удерживая целевой ДРР и выкуп и позволяя вести больше селлеров без роста ручной работы.</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n">
@@ -7448,6 +8444,11 @@
           <t>Производитель готовой еды: кухня работает на полную, а прибыль тает к ночи — сколько денег уезжает в мусорный бак вместе с непроданными за день порциями?</t>
         </is>
       </c>
+      <c r="H200" s="3" t="inlineStr">
+        <is>
+          <t>Производитель готовой еды: ИИ по продажам точек, дням недели и сроку годности рассчитывает объём готовки на каждую точку, сокращая вечерние списания непроданных порций и повышая маржу.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
@@ -7483,6 +8484,11 @@
           <t>Хостел: койки заняты почти всегда, а денег в обрез — правда ли, что низкий чек и вечная текучка гостей не оставляют прибыли после уборки и стирки?</t>
         </is>
       </c>
+      <c r="H201" s="3" t="inlineStr">
+        <is>
+          <t>Хостел: ИИ по графику заездов и выездов планирует смены уборки и стирки под реальную загрузку, сокращая переплату за простой персонала и поднимая маржу с койко-места.</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
@@ -7518,6 +8524,11 @@
           <t>Частный детский сад: группы укомплектованы, очередь на входе, а прибыли почти нет — куда уходит абонентская плата, если зарплаты и питание дорожают быстрее ценника?</t>
         </is>
       </c>
+      <c r="H202" s="3" t="inlineStr">
+        <is>
+          <t>Частный детский сад: ИИ планирует меню и оптимизирует закупки продуктов по ценам поставщиков и нормам питания, снижая себестоимость питания и удерживая маржу при фиксированной оплате.</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
@@ -7553,6 +8564,11 @@
           <t>Концертная площадка: аншлаг в пятницу, а вторник и среда — пустой зал под тем же светом и охраной — сколько прибыли сжигают простаивающие даты?</t>
         </is>
       </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>Концертная площадка: ИИ по спросу города и истории продаж подбирает артистов и события под пустые даты, заполняя простаивающие будни и покрывая постоянные расходы на аренду и охрану.</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
@@ -7580,12 +8596,17 @@
       </c>
       <c r="F204" s="3" t="inlineStr">
         <is>
-          <t>Собираем заявки клиентов, квалифицируем и подбираем варианты, ведём переговоры и показы, сопровождаем сделку до подписания, получаем комиссию за закрытие.</t>
+          <t>Открываем клиенту брокерский счёт, проводим квалификацию, даём доступ к торгам на бирже, принимаем и исполняем заявки, храним активы, готовим отчётность и удерживаем комиссию с оборота.</t>
         </is>
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
           <t>Брокерская компания: лидов гора, менеджеры в мыле, а платят только за закрытые сделки — сколько выручки утекает с клиентами, до которых руки так и не дошли?</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr">
+        <is>
+          <t>Брокерская компания: ИИ скорит поток лидов по вероятности открытия счёта и оборота, направляя менеджеров на горячих клиентов первыми и повышая долю закрытых сделок из входящего потока.</t>
         </is>
       </c>
     </row>
@@ -7623,6 +8644,11 @@
           <t>Онлайн-магазин косметики: крем заканчивается ровно через месяц, клиент готов купить снова — почему за добавкой он идёт не к вам, и сколько на этом теряется LTV?</t>
         </is>
       </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>Онлайн-магазин косметики: ИИ по составу заказа и расходу прогнозирует дату, когда средство заканчивается, и шлёт напоминание о повторной покупке, возвращая клиента и повышая LTV.</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
@@ -7658,6 +8684,11 @@
           <t>Компания по кибербезопасности: спрос огромный, специалистов не хватает — почему выручка обрывается на сдаче проекта, вместо того чтобы капать постоянно?</t>
         </is>
       </c>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>Компания по кибербезопасности: ИИ непрерывно выявляет аномалии в трафике и логах клиента между аудитами, превращая разовые проекты в абонентский мониторинг и добавляя повторяемую выручку.</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n">
@@ -7693,6 +8724,11 @@
           <t>Магазин оптики: поток на проверку зрения есть, а касса скромная — сколько клиентов уходят с рецептом в руке, чтобы заказать очки где-то дешевле?</t>
         </is>
       </c>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>Магазин оптики: ИИ-конфигуратор виртуально примеряет оправы по фото лица и подбирает тип линз под рецепт, повышая конверсию из проверки зрения в покупку прямо на месте.</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
@@ -7728,6 +8764,11 @@
           <t>Агентство хоумстейджинга: оформленная квартира продаётся быстрее и дороже, а склад с мебелью простаивает между заказами — сколько прибыли лежит мёртвым грузом?</t>
         </is>
       </c>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>Агентство хоумстейджинга: ИИ планирует ротацию мебели и декора между объектами по графику проектов, повышая оборачиваемость склада реквизита и сокращая простой мёртвого груза между заказами.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
@@ -7763,6 +8804,11 @@
           <t>Сервис выгула собак: заявок много, а выгульщик успевает мало — сколько прибыли съедают пробки и километры между клиентами на разных концах города?</t>
         </is>
       </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>Сервис выгула собак: ИИ группирует заявки по районам и строит маршруты выгульщиков, сокращая время на дорогу между адресами и увеличивая число прогулок в день на человека.</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
@@ -7798,6 +8844,11 @@
           <t>Охрана труда на аутсорсе: клиент платит абонентку за спокойствие, а вы тонете в бумагах — сколько времени уходит на ручное заполнение журналов вместо новых договоров?</t>
         </is>
       </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>Охрана труда на аутсорсе: ИИ извлекает данные из документов клиента и автоматически заполняет журналы, приказы и инструктажи, сокращая ручной ввод и позволяя вести больше договоров на абонентке.</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
@@ -7805,7 +8856,7 @@
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>Студия пилатеса</t>
+          <t>Студия лазерной эпиляции</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
@@ -7815,22 +8866,27 @@
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>Абонентская подписка</t>
+          <t>Оплата за услугу</t>
         </is>
       </c>
       <c r="E211" s="3" t="inlineStr">
         <is>
-          <t>Студия пилатеса: как удержать подписчиков и заполнить реформеры, если оплаченный абонемент ещё не значит, что клиент ходит?</t>
+          <t>Студия лазерной эпиляции: как догружать простаивающий аппарат между сеансами и доводить клиента до конца курса из шести-восьми процедур?</t>
         </is>
       </c>
       <c r="F211" s="3" t="inlineStr">
         <is>
-          <t>Продаём подписку, ставим расписание групп на реформерах, ведём занятия по уровням, следим за посещаемостью, напоминаем о тренировках, продлеваем абонементы.</t>
+          <t>Мы консультируем и тестируем реакцию кожи, бреем зону, ведём клиента по курсу с интервалом в месяц, отрабатываем аппаратом, записываем на следующий сеанс и напоминаем не бросить курс.</t>
         </is>
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>Студия пилатеса: подписки оплачены, а залы полупустые — правда ли, что клиент, который перестал ходить, уже одной ногой ушёл, а его отток вы заметите слишком поздно?</t>
+          <t>Студия лазерной эпиляции: можно ли отбить дорогой аппарат, если клиент пропадает после второй процедуры из восьми оплаченных?</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>Студия лазерной эпиляции: ИИ по графику курса выявляет клиентов, бросающих процедуры после второго сеанса, и запускает напоминания и стимулы, доводя курс до конца и загружая аппарат.</t>
         </is>
       </c>
     </row>
@@ -7868,6 +8924,11 @@
           <t>Шиномонтаж: в сезон переобувки очередь на улицу и хаос, а между пиками бокс пустует — сколько прибыли теряется на том, что весь год зажат в две недели?</t>
         </is>
       </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>Шиномонтаж: динамическое ценообразование слотов по истории записей и погоде — скидки в межсезон и будни, премия в пик; сглаживаем очередь и грузим бокс в мёртвые месяцы.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n">
@@ -7903,6 +8964,11 @@
           <t>Хостинг-провайдер: почему выручка по подписке вроде стабильна, а прибыль утекает в ночную поддержку и клиентов, что уходят к конкуренту за пятьдесят рублей?</t>
         </is>
       </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>Хостинг-провайдер: модель оттока по логам нагрузки, тикетам и истории платежей предсказывает несостоявшиеся продления за месяц — триггерный оффер и апселл тарифа снижают отток и растят ARPU.</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n">
@@ -7910,7 +8976,7 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>Апарт-отель</t>
+          <t>Глэмпинг</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
@@ -7925,17 +8991,22 @@
       </c>
       <c r="E214" s="3" t="inlineStr">
         <is>
-          <t>Апарт-отель: как поднять загрузку в будни и низкий сезон и не отдавать маржу на комиссиях агрегаторов бронирования?</t>
+          <t>Глэмпинг: как выровнять загрузку шатров вне сезона и удержать маржу, когда доход держится на трёх летних месяцах?</t>
         </is>
       </c>
       <c r="F214" s="3" t="inlineStr">
         <is>
-          <t>Принимаем брони с площадок, заселяем и выдаём ключи, убираем номера между гостями, отвечаем на вопросы жильцов, докручиваем допродажи и обрабатываем отзывы.</t>
+          <t>Мы принимаем брони, готовим шатры и постель к заезду, топим печь и баню, встречаем гостей, кормим завтраком, водим на активности, а после выезда убираем и снова выставляем даты.</t>
         </is>
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>Апарт-отель: куда утекает прибыль, если номера почти всегда заняты, а после комиссий агрегаторов, уборки и простоев в будни касса всё равно тонкая?</t>
+          <t>Глэмпинг: куда утекает годовая прибыль, если шатры забиты в июле под ноль, а к октябрю стоят пустыми?</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>Глэмпинг: ИИ перераспределяет рекламный бюджет по данным прошлых броней и сезонности, таргетируя будни и межсезон — ниже стоимость брони и выше загрузка шатров в октябре.</t>
         </is>
       </c>
     </row>
@@ -7973,6 +9044,11 @@
           <t>Магазин цифровых товаров: правда ли, что продажа без склада и логистики — лёгкие деньги, если фрод, возвраты и мёртвые остатки ключей едят всю наценку?</t>
         </is>
       </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>Магазин цифровых товаров: антифрод-модель по параметрам заказа, платежа и устройства помечает рисковые покупки до выдачи ключа — меньше чарджбеков и возвратов, наценку не съедает фрод.</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n">
@@ -8008,6 +9084,11 @@
           <t>Управляющая компания активами: что скрывается за красивой доходностью в презентации, если половина времени управляющих уходит на отчёты, а не на решения по портфелю?</t>
         </is>
       </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>Управляющая компания активами: ИИ автоформирует клиентскую отчётность и комментарии по портфелю из данных позиций и сделок — управляющие тратят часы не на отчёты, а на решения, и ведут больше клиентов.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n">
@@ -8043,6 +9124,11 @@
           <t>Видеопродакшн: сколько денег сгорает на бесконечных кругах правок и переносах съёмок, пока смена оплачена, а готового ролика всё ещё нет?</t>
         </is>
       </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>Видеопродакшн: ИИ собирает черновой монтаж, чистит звук, ставит цвет и субтитры по отснятому материалу — монтажёр отдаёт первую версию быстрее, меньше кругов правок и простоев смены.</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n">
@@ -8070,12 +9156,17 @@
       </c>
       <c r="F218" s="3" t="inlineStr">
         <is>
-          <t>Зовём на пробное занятие, набираем группы по возрастам, ведём расписание педагогов, продаём абонементы, напоминаем о занятиях и удерживаем родителей.</t>
+          <t>Зовём на пробное занятие, набираем группы по возрастам, ставим педагогов и расписание, проводим развивающие занятия, отслеживаем прогресс детей, показываем результат родителям, продаём и продлеваем абонементы.</t>
         </is>
       </c>
       <c r="G218" s="3" t="inlineStr">
         <is>
           <t>Детский развивающий центр: почему после блестящего пробного занятия половина родителей не покупает абонемент, а группы в будни днём стоят полупустыми?</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>Детский развивающий центр: модель по итогам пробного и анкете предсказывает, кто не купит абонемент, и запускает персональный оффер и звонок педагога — конверсия пробного в абонемент растёт.</t>
         </is>
       </c>
     </row>
@@ -8113,6 +9204,11 @@
           <t>Молочная ферма: куда исчезает прибыль, если коровы доятся, молоко льётся, а переработчик диктует цену и снимает за каждую десятую процента жирности?</t>
         </is>
       </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>Молочная ферма: ИИ по данным надоев, активности и ветучёта каждой коровы ловит мастит и спад рациона на ранней стадии — выше надой и жирность, меньше выбраковки и потерь на болезнях.</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n">
@@ -8148,6 +9244,11 @@
           <t>Агентство домашнего персонала: правда ли, что работа — просто свести семью и няню, если после первой встречи они договариваются напрямую и агентство остаётся без комиссии?</t>
         </is>
       </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>Агентство домашнего персонала: ИИ сопоставляет запрос семьи с профилями кандидатов по опыту, графику и отзывам — точнее первый подбор и быстрая замена, семьи реже уходят на прямую оплату.</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n">
@@ -8183,6 +9284,11 @@
           <t>Студия йоги: почему проданный абонемент — ещё не деньги, если человек сходил три раза, бросил и не продлил, а зал в обед пустует?</t>
         </is>
       </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>Студия йоги: модель по частоте визитов и паузам предсказывает, кто бросает после трёх занятий — автонапоминание и персональный оффер возвращают клиента и повышают продление абонементов.</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n">
@@ -8218,6 +9324,11 @@
           <t>Аутсорсинговый отдел продаж: что ломается первым, когда клиент платит за подписку, а звонки уходят вхолостую и он винит вас в слабых лидах со своего же рынка?</t>
         </is>
       </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>Аутсорсинговый отдел продаж: скоринг лидов из базы клиента по отклику и профилю расставляет очередь звонков — менеджеры работают по горячим, меньше вхолостую, выше конверсия во встречи на том же штате.</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n">
@@ -8253,6 +9364,11 @@
           <t>Компания по приёмке квартир: куда утекает выручка, если эксперт объезжает три квартиры в день, а на составление актов и дефектовку вечером уходят ещё часы?</t>
         </is>
       </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>Компания по приёмке квартир: ИИ по фото, замерам и заметкам с объекта автоформирует акт дефектов и претензию застройщику — вечерняя бумажная работа исчезает, эксперт делает больше приёмок в день.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n">
@@ -8288,6 +9404,11 @@
           <t>Аптечная сеть: сколько прибыли лежит на полках в виде препаратов, которые спишутся по сроку раньше, чем их кто-нибудь спросит?</t>
         </is>
       </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>Аптечная сеть: ИИ прогнозирует спрос по SKU и срокам годности, корректирует заказ и перебрасывает предликвид между точками — списания по просрочке падают, оборачиваемость выше.</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n">
@@ -8323,6 +9444,11 @@
           <t>Молочный завод: правда ли, что завод зарабатывает на объёме, если недозагруженные линии, возвраты из сетей и короткий срок годности съедают всю рентабельность партии?</t>
         </is>
       </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>Молочный завод: прогноз спроса по сетям и SKU планирует объём розлива под реальные заказы и сроки — линии загружены ровнее, возвратов по истёкшему сроку меньше.</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n">
@@ -8358,6 +9484,11 @@
           <t>Театральная студия: куда утекает касса, если премьеры собирают аншлаг, а на будних показах полупустой зал платит за тот же свет, аренду и труппу?</t>
         </is>
       </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>Театральная студия: рекомендательный движок допродаёт по истории покупок буфет, мерч и платные курсы актёрского каждому зрителю — средний чек показа растёт без зависимости от одного аншлага.</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n">
@@ -8393,6 +9524,11 @@
           <t>Спортивная секция: почему после сезона и соревнований половина группы отваливается, а тренер получает за полупустой зал столько же времени, сколько за полный?</t>
         </is>
       </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>Спортивная секция: модель оттока по посещаемости, оплатам и результатам ловит детей, готовых уйти после сезона — тренер получает сигнал и сценарий удержания, группы не пустеют.</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n">
@@ -8428,6 +9564,11 @@
           <t>Банкетный зал: сколько теряет заведение на пустых будних вечерах и сорванных бронях, если суббота расписана на год вперёд, а понедельник стоит тёмным?</t>
         </is>
       </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>Банкетный зал: динамические цены и пакеты по спросу на даты — премия за субботу, скидки и депозит на будни — грузим пустые вечера и поднимаем маржу заказа, меньше сорванных броней.</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
@@ -8463,6 +9604,11 @@
           <t>Автошкола: куда утекают деньги, если группа набрана и оплачена, а до экзамена доезжает половина, и машины инструкторов простаивают в неудобные часы?</t>
         </is>
       </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>Автошкола: ИИ распределяет учеников по инструкторам, машинам и площадке под свободные часы и уровень — простой машин в неудобное время падает, группы едут ровнее к экзамену.</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n">
@@ -8498,6 +9644,11 @@
           <t>Автомойка: почему выручка скачет вместе с погодой, если в ливень очередь на час, а в сухой день мойщики и боксы стоят без дела?</t>
         </is>
       </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>Автомойка: прогноз почасовой загрузки по погоде и истории чеков ставит нужное число мойщиков и запускает промо в сухие часы — меньше потерянных машин в очередь и простоя боксов.</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">
@@ -8533,6 +9684,11 @@
           <t>Редакция корпоративных медиа: сколько маржи сгорает в кругах согласований, если статья готова за день, а заказчик правит её три недели по абзацу?</t>
         </is>
       </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>Редакция корпоративных медиа: RAG-ассистент на базе бренд-гайда и утверждённых текстов клиента готовит черновики в его тональности — меньше кругов согласований, редактор ведёт больше клиентов.</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n">
@@ -8568,6 +9724,11 @@
           <t>Финансовый консультант: что скрывается за success fee, если на сборку персонального плана уходят дни, а клиент внедряет советы через раз и результат не гарантирован?</t>
         </is>
       </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>Финансовый консультант: ИИ собирает черновик персонального финплана из данных о доходах, долгах и целях клиента — консультант правит, а не пишет с нуля, и ведёт больше клиентов на том же времени.</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n">
@@ -8603,6 +9764,11 @@
           <t>Интернет-провайдер: куда утекает прибыль, если абонент платит копеечную абонплату, а один выезд бригады на обрыв съедает выручку с него за полгода?</t>
         </is>
       </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>Интернет-провайдер: модель оттока по авариям, скорости и обращениям выделяет абонентов, готовых уйти к демпингующему конкуренту — превентивный оффер и апселл допуслуг удерживают их и растят чек.</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n">
@@ -8638,6 +9804,11 @@
           <t>Оценочная компания недвижимости: правда ли, что оценщик зарабатывает на выезде, если больше половины времени уходит на подбор аналогов и оформление толстого отчёта под банк?</t>
         </is>
       </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>Оценочная компания недвижимости: ИИ подбирает объекты-аналоги из баз объявлений и сделок и предзаполняет отчёт — оценщик тратит время не на поиск аналогов, а на проверку, отчётов в месяц больше.</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n">
@@ -8673,6 +9844,11 @@
           <t>Print-on-demand бренд: сколько наценки съедают возвраты и брак печати, если склада нет, но каждый неугаданный размер и кривой оттиск — это чистый убыток?</t>
         </is>
       </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>Print-on-demand бренд: ИИ-рекомендатель размера по параметрам покупателя и таблице посадки подсказывает верный размер до заказа — возвраты по размеру падают, повторные покупки растут.</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n">
@@ -8708,6 +9884,11 @@
           <t>Магазин автозапчастей: куда вмораживается прибыль, если ходовые фильтры разбирают за день, а полки забиты деталями, которые ждут своего покупателя третий год?</t>
         </is>
       </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>Магазин автозапчастей: прогноз спроса по SKU, VIN-запросам и сезону задаёт точку заказа ходовых и вычищает неликвид — оборачиваемость склада выше, меньше денег заморожено в мёртвых полках.</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n">
@@ -8743,6 +9924,11 @@
           <t>Контакт-центр на аутсорсе: что ломается первым, когда клиент платит за подписку, а половина смены операторов уходит на найм и обучение вечно текучих новичков?</t>
         </is>
       </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>Контакт-центр на аутсорсе: ИИ-ассистент берёт типовые чаты и звонки и подсказывает оператору ответ — одна смена держит больше линий, экономика не проседает на зарплатах и обучении новичков.</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n">
@@ -8778,6 +9964,11 @@
           <t>Пункт выдачи заказов: правда ли, что это лёгкий пассивный бизнес, если комиссия копеечная, а очереди на примерку и гора возвратов держатся на одном сотруднике?</t>
         </is>
       </c>
+      <c r="H238" s="3" t="inlineStr">
+        <is>
+          <t>Пункт выдачи заказов: ИИ прогнозирует пики выдач, примерок и возвратов по данным поставок и истории заказов и ставит сотрудника под час пик — меньше очередей и брошенных выкупов.</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n">
@@ -8805,12 +9996,17 @@
       </c>
       <c r="F239" s="3" t="inlineStr">
         <is>
-          <t>Закладываем инкубацию, выращиваем поголовье на кормах, следим за падежом и ветеринарией, собираем и сортируем яйцо, забиваем и фасуем, развозим по сетям.</t>
+          <t>Закладываем яйцо в инкубатор, выращиваем поголовье на кормах, следим за падежом и ветеринарией, собираем и сортируем яйцо у несушек либо забиваем и разделываем бройлера, фасуем и развозим по сетям.</t>
         </is>
       </c>
       <c r="G239" s="3" t="inlineStr">
         <is>
           <t>Птицефабрика: куда утекает рентабельность, если птица растёт по графику, а скачок цены на корма и падёж в одном птичнике съедают маржу всей партии?</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>Птицефабрика: предиктивный контроль микроклимата и оборудования птичников по датчикам вентиляции, поения и температуры предупреждает аварии и падёж до вспышки — сохраняем выход партии.</t>
         </is>
       </c>
     </row>
@@ -8848,6 +10044,11 @@
           <t>Гончарная мастерская: почему прибыль тает между занятиями, если группы идут по выходным, а печь, глина и мастер простаивают всю неделю в ожидании обжига?</t>
         </is>
       </c>
+      <c r="H240" s="3" t="inlineStr">
+        <is>
+          <t>Гончарная мастерская: ИИ оптимизирует сетку мастер-классов и загрузку печи, группируя обжиги и заполняя будни по спросу — печь и мастер не простаивают всю неделю, выше выручка со слота.</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n">
@@ -8883,6 +10084,11 @@
           <t>Мясоперерабатывающее предприятие: сколько прибыли уходит в обрезь и возвраты, если каждый процент выхода с туши и день срока годности решают, в плюсе вы или в минусе?</t>
         </is>
       </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>Мясоперерабатывающее предприятие: компьютерное зрение на обвалке контролирует выход и жиловку по каждой туше — ловим потери в обрезь и брак раньше, каждый процент выхода остаётся в марже.</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n">
@@ -8918,6 +10124,11 @@
           <t>Краудфандинговая платформа: куда утекает выручка, если комиссия капает только с успешных сборов, а большинство кампаний глохнет на полпути и не доходит до цели?</t>
         </is>
       </c>
+      <c r="H242" s="3" t="inlineStr">
+        <is>
+          <t>Краудфандинговая платформа: скоринг новых кампаний по данным прошлых сборов — динамика первых дней, структура наград, активность автора — направляет поддержку на спасаемые проекты; растёт доля доходящих до цели и объём комиссии.</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n">
@@ -8953,6 +10164,11 @@
           <t>Реабилитационный центр: почему расписание врачей забито, а выручка стоит, если половина пациентов бросает курс после третьего занятия?</t>
         </is>
       </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>Реабилитационный центр: модель на данных посещаемости и динамики восстановления предсказывает срыв курса после 2–3 занятий и запускает напоминания — доля доходящих до конца курса выше, кресла специалистов загружены.</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n">
@@ -8988,6 +10204,11 @@
           <t>SaaS-компания: что скрывается за красивым ростом регистраций, если через три месяца платит меньше половины, а MRR утекает быстрее, чем растёт?</t>
         </is>
       </c>
+      <c r="H244" s="3" t="inlineStr">
+        <is>
+          <t>SaaS-компания: прогноз оттока по продуктовой телеметрии — частоте входов, глубине использования фич, тикетам — находит аккаунты, уходящие на 2–3-м месяце, и триггерит удержание до продления; отток MRR снижается.</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n">
@@ -9023,6 +10244,11 @@
           <t>Музыкальная школа: куда утекает прибыль, если педагоги на окладе, а треть уроков срывается из-за отмен и «окон» в расписании?</t>
         </is>
       </c>
+      <c r="H245" s="3" t="inlineStr">
+        <is>
+          <t>Музыкальная школа: ИИ оптимизирует расписание педагогов и мгновенно переставляет отменённые уроки на учеников из листа ожидания, закрывая «окна» — доля сорванных занятий падает, загрузка окладных педагогов растёт.</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n">
@@ -9058,6 +10284,11 @@
           <t>Компания по установке солнечных панелей: почему заявок много, а денег мало, если между «посчитайте мне» и подписанным договором проходят месяцы сомнений?</t>
         </is>
       </c>
+      <c r="H246" s="3" t="inlineStr">
+        <is>
+          <t>Компания по установке солнечных панелей: по замеру, инсоляции и тарифам ИИ за минуты собирает персональное КП с расчётом окупаемости и графиком экономии — цикл сделки короче, конверсия из «посчитайте» в договор выше.</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n">
@@ -9093,6 +10324,11 @@
           <t>Виртуальный офис и секретарский сервис: сколько абонентов теряется, когда секретарь занят на другой линии, а звонящий кладёт трубку и уходит к конкуренту?</t>
         </is>
       </c>
+      <c r="H247" s="3" t="inlineStr">
+        <is>
+          <t>Виртуальный офис и секретарский сервис: голосовой ИИ-ассистент принимает параллельные звонки от имени каждого абонента, фиксирует и переадресует обращения — входящие не теряются на занятой линии, поток масштабируется без роста штата секретарей.</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n">
@@ -9128,6 +10364,11 @@
           <t>Салон проката платьев: правда ли, что главный убыток — не порванное платье, а недели простоя между выпускным сезоном и свадьбами?</t>
         </is>
       </c>
+      <c r="H248" s="3" t="inlineStr">
+        <is>
+          <t>Салон проката платьев: динамическое ценообразование по сезону, размеру и загрузке гардероба поднимает аренду в пик и стимулирует бронь в межсезонье скидками на простаивающие модели — оборачиваемость и выручка низкого сезона растут.</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n">
@@ -9163,6 +10404,11 @@
           <t>Загородный клуб: куда уходит прибыль, когда территория красивая, а с понедельника по четверг домики пустуют, но персонал всё равно на смене?</t>
         </is>
       </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>Загородный клуб: ИИ перераспределяет рекламный бюджет и ретаргетит прошлых гостей под будние заезды и небанкетные даты — номера и площадки грузятся с понедельника по четверг, стоимость брони снижается.</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n">
@@ -9198,6 +10444,11 @@
           <t>Автосалон подержанных автомобилей: сколько денег замораживает каждая машина, что стоит на площадке лишний месяц, пока капитал висит в неликвиде?</t>
         </is>
       </c>
+      <c r="H250" s="3" t="inlineStr">
+        <is>
+          <t>Автосалон подержанных автомобилей: ИИ по рыночным ценам и истории просмотров задаёт цену каждой машины и вовремя снижает по «зависшим» — средний срок на площадке падает, меньше капитала заморожено в неликвиде.</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n">
@@ -9233,6 +10484,11 @@
           <t>Хлебозавод: почему план по объёму выполнен, а прибыль тает, если каждая пятая буханка возвращается из магазина и уходит в списание?</t>
         </is>
       </c>
+      <c r="H251" s="3" t="inlineStr">
+        <is>
+          <t>Хлебозавод: прогноз спроса по каждой торговой точке и дню недели на истории продаж, погоде и праздниках задаёт объём выпечки и развоза — возвраты и списания снижаются без пустых полок к вечернему пику.</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n">
@@ -9268,6 +10524,11 @@
           <t>Агентство личного бренда: что ломается первым, когда клиентов становится больше, а продюсер физически не может вести десять блогов одновременно?</t>
         </is>
       </c>
+      <c r="H252" s="3" t="inlineStr">
+        <is>
+          <t>Агентство личного бренда: генеративный ИИ по транскриптам съёмок эксперта готовит черновики постов, нарезки и сценарии рубрик — один продюсер ведёт больше блогов, себестоимость контента падает.</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n">
@@ -9295,12 +10556,17 @@
       </c>
       <c r="F253" s="3" t="inlineStr">
         <is>
-          <t>Зарыбляем садки мальком, кормим по графику, следим за кислородом и температурой воды, сортируем рыбу по навеске, отлавливаем товарную и поставляем покупателям.</t>
+          <t>Зарыбляем водоёмы мальком, подращиваем и кормим по графику, контролируем кислород, температуру и здоровье рыбы, сортируем по навеске, отлавливаем товарную и поставляем покупателям.</t>
         </is>
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
           <t>Рыбное хозяйство: куда утекает прибыль, если корм дорожает, часть малька не доживает до товарной навески, а цену на вылов диктует рынок?</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr">
+        <is>
+          <t>Рыбное хозяйство: модель по данным о температуре, кислороде, навеске и кормлении прогнозирует набор товарной массы и риск падёжа, оптимизируя график корма — конверсия корма (FCR) улучшается, отход малька снижается.</t>
         </is>
       </c>
     </row>
@@ -9338,6 +10604,11 @@
           <t>Subscription box сервис: почему первая коробка радует, а к третьей половина подписчиков отписывается, и стоимость привлечения так и не отбивается?</t>
         </is>
       </c>
+      <c r="H254" s="3" t="inlineStr">
+        <is>
+          <t>Subscription box сервис: рекомендательная система по анкете и реакциям на прошлые коробки — что оставили, что вернули — подбирает наполнение следующего набора; отписки после третьей коробки снижаются, растёт число продлений.</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n">
@@ -9345,7 +10616,7 @@
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Музыкальный лейбл</t>
+          <t>Аквапарк</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
@@ -9355,22 +10626,27 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>Продажи прав / revenue share</t>
+          <t>Билеты + дополнительные продажи</t>
         </is>
       </c>
       <c r="E255" s="3" t="inlineStr">
         <is>
-          <t>Музыкальный лейбл: как выстроить поток релизов и не зависеть от одного хита, если гонорары платятся вперёд, а роялти капают месяцами?</t>
+          <t>Аквапарк: как сгладить зависимость выручки от погоды и разгрузить пропускную способность горок в пиковые часы выходных?</t>
         </is>
       </c>
       <c r="F255" s="3" t="inlineStr">
         <is>
-          <t>Ищем артистов, подписываем контракт, продюсируем и записываем треки, размещаем на площадках, продвигаем релизы в плейлистах и делим доход от стримов по договору.</t>
+          <t>Мы продаём билеты и браслеты, запускаем посетителей потоками, следим за горками и чашами, дежурим спасателями, крутим оборот шкафчиков, кормим в кафе и закрываем смену уборкой и обеззараживанием воды.</t>
         </is>
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>Музыкальный лейбл: что скрывается за миллионами прослушиваний, если аванс артисту уже выплачен, а стриминговые роялти отбивают вложения только через год?</t>
+          <t>Аквапарк: правда ли, что один дождливый выходной съедает выручку недели, а солнечный день упирается в очередь на горку?</t>
+        </is>
+      </c>
+      <c r="H255" s="3" t="inlineStr">
+        <is>
+          <t>Аквапарк: компьютерное зрение считает очереди и загрузку чаш в реальном времени и подсказывает перераспределение потоков и открытие горок — время ожидания в пик выходных падает, пропускная способность растёт.</t>
         </is>
       </c>
     </row>
@@ -9408,6 +10684,11 @@
           <t>Магазин бытовой техники: сколько теряет продавец, когда покупатель щупает холодильник у него на витрине, а оформляет заказ в приложении по дороге домой?</t>
         </is>
       </c>
+      <c r="H256" s="3" t="inlineStr">
+        <is>
+          <t>Магазин бытовой техники: рекомендательный ассистент у продавца по товару и профилю покупателя предлагает релевантные допы, установку и расширенную гарантию — средний чек и маржа растут даже при цене «как на маркетплейсе».</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n">
@@ -9443,6 +10724,11 @@
           <t>Компания по монтажу систем безопасности: почему после сдачи объекта прибыль обнуляется, если смонтировал, получил оплату и снова ищешь следующего клиента с нуля?</t>
         </is>
       </c>
+      <c r="H257" s="3" t="inlineStr">
+        <is>
+          <t>Компания по монтажу систем безопасности: предиктивное обслуживание по телеметрии установленных камер и датчиков заранее выявляет сбои и сам предлагает клиенту сервис — доля объектов на постоянном обслуживании и повторная выручка растут.</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n">
@@ -9478,6 +10764,11 @@
           <t>Кондитерское производство: куда девается маржа, если под 8 марта заказы не успеваешь выполнить, а в будни кондитеры простаивают, а продукты портятся?</t>
         </is>
       </c>
+      <c r="H258" s="3" t="inlineStr">
+        <is>
+          <t>Кондитерское производство: прогноз нагрузки по датам и праздникам планирует смены, временных кондитеров под пики и закупку скоропорта — заказы к 8 марта выполняются, простой в будни и порча продуктов снижаются.</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n">
@@ -9513,6 +10804,11 @@
           <t>Танцевальная школа: почему залы пустуют днём и переполнены вечером, а абонементы, купленные в сентябре, к ноябрю никто не продлевает?</t>
         </is>
       </c>
+      <c r="H259" s="3" t="inlineStr">
+        <is>
+          <t>Танцевальная школа: модель по посещаемости выявляет учеников, теряющих мотивацию после первого месяца, и запускает персональные касания до окончания абонемента — продлений больше, отток к ноябрю ниже.</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n">
@@ -9548,6 +10844,11 @@
           <t>Компания по подбору автомобилей: сколько сделок срывается, пока специалист неделю мотается по осмотрам, а клиент тем временем сам покупает первую попавшуюся машину?</t>
         </is>
       </c>
+      <c r="H260" s="3" t="inlineStr">
+        <is>
+          <t>Компания по подбору автомобилей: ИИ по критериям клиента отбирает подходящие объявления и авто-проверяет историю и чистоту, отсекая пустые выезды — специалист доводит больше подборов до сделки за то же время.</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n">
@@ -9583,6 +10884,11 @@
           <t>Ломбард: правда ли, что деньги делаются не на процентах по займу, а на витрине с невыкупленными вещами, которые месяцами лежат без покупателя?</t>
         </is>
       </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>Ломбард: ИИ оценивает принесённый залог по фото и рыночным аналогам, прогнозируя ликвидность и цену реализации — меньше ошибок оценки, витрина оборачивается быстрее, касса не зависает в невыкупленном неликвиде.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n">
@@ -9618,6 +10924,11 @@
           <t>Туроператор: куда утекает прибыль сезона, если непроданное кресло в чартере и пустой номер в отеле уже оплачены, а вылет через три дня?</t>
         </is>
       </c>
+      <c r="H262" s="3" t="inlineStr">
+        <is>
+          <t>Туроператор: динамическое ценообразование по остаткам мест и дате вылета уценяет непроданные кресла в чартере и номера перед сгоранием — доля распроданных блоков растёт, потери на «горящих» местах снижаются.</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n">
@@ -9645,12 +10956,17 @@
       </c>
       <c r="F263" s="3" t="inlineStr">
         <is>
-          <t>Придумываем концепт, прототипируем механики, разрабатываем и тестируем игру, выпускаем в магазины, поддерживаем обновлениями и зарабатываем на продажах и внутриигровых покупках.</t>
+          <t>Придумываем концепт, прототипируем механики, разрабатываем и тестируем игру, готовим маркетинг и комьюнити, выпускаем в магазины и удерживаем игроков живыми обновлениями.</t>
         </is>
       </c>
       <c r="G263" s="3" t="inlineStr">
         <is>
           <t>Студия разработки видеоигр: что будет со студией, если два года команда горит на одном проекте, а игроки уходят из игры через неделю после релиза?</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr">
+        <is>
+          <t>Студия разработки видеоигр: модель по телеметрии сессий находит уровни и дни, где игроки бросают игру на первой неделе, и приоритизирует правки в обновлениях — ранее удержание растёт.</t>
         </is>
       </c>
     </row>
@@ -9688,6 +11004,11 @@
           <t>Винный магазин: что скрывается за полными полками, если оборот делают три ходовые бутылки, а дорогая коллекция месяцами стоит замороженными деньгами?</t>
         </is>
       </c>
+      <c r="H264" s="3" t="inlineStr">
+        <is>
+          <t>Винный магазин: ИИ-сомелье по чекам и поводу покупателя рекомендует вино и гастропары, подсвечивая дорогие и редкие позиции — средний чек растёт, коллекция распродаётся, а не пылится на полке.</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n">
@@ -9723,6 +11044,11 @@
           <t>Агентство маркетинговых исследований: почему проект прибыльный на бумаге, если половину гонорара съедают недели ручной расшифровки анкет и сведения таблиц?</t>
         </is>
       </c>
+      <c r="H265" s="3" t="inlineStr">
+        <is>
+          <t>Агентство маркетинговых исследований: ИИ транскрибирует и резюмирует интервью и открытые анкеты, сводя ответы в темы и выводы — недели ручной расшифровки сокращаются, агентство берёт больше проектов теми же людьми.</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n">
@@ -9758,6 +11084,11 @@
           <t>Маркетплейс услуг: куда утекает комиссия, если после первого заказа клиент и мастер обмениваются телефонами и следующие сделки проходят мимо площадки?</t>
         </is>
       </c>
+      <c r="H266" s="3" t="inlineStr">
+        <is>
+          <t>Маркетплейс услуг: ИИ выявляет аномалии в переписке и заказах — обмен контактами и увод сделок мимо площадки — и вовремя удерживает клиента бонусами; доля повторных сделок внутри платформы и комиссия растут.</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n">
@@ -9793,6 +11124,11 @@
           <t>Издательство: правда ли, что главный убыток — не провальная книга, а раздутый тираж хорошего автора, половина которого вернётся из магазинов на склад?</t>
         </is>
       </c>
+      <c r="H267" s="3" t="inlineStr">
+        <is>
+          <t>Издательство: прогноз спроса по жанру, автору и предзаказам подбирает оптимальный тираж и допечатку — возвраты из магазинов и замороженные на складе остатки снижаются без дефицита ходовых книг.</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n">
@@ -9828,6 +11164,11 @@
           <t>Агентство корпоративных поездок: сколько маржи съедает один отменённый рейс, когда менеджер полночи вручную пересобирает маршрут командированного за те же деньги?</t>
         </is>
       </c>
+      <c r="H268" s="3" t="inlineStr">
+        <is>
+          <t>Агентство корпоративных поездок: ИИ извлекает данные из билетов, счетов и travel-политик и авто-готовит перевыставление и отчётность при заменах рейсов — менеджер обрабатывает больше командировок без ночной ручной пересборки.</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n">
@@ -9863,6 +11204,11 @@
           <t>Прокат оборудования для мероприятий: куда уходит прибыль, если дорогой комплект света бронируют только по субботам, а всю неделю он лежит на складе мёртвым грузом?</t>
         </is>
       </c>
+      <c r="H269" s="3" t="inlineStr">
+        <is>
+          <t>Прокат оборудования для мероприятий: ИИ оптимизирует календарь броней и комплектацию звука и света, предлагая будние тарифы под простаивающие комплекты — оборачиваемость дорогого оборудования и загрузка в будни растут.</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n">
@@ -9898,6 +11244,11 @@
           <t>Компания по переработке отходов: почему объёмы приёмки растут, а прибыль нет, если половина привезённого — грязь и брак, а цена на вторсырьё падает без предупреждения?</t>
         </is>
       </c>
+      <c r="H270" s="3" t="inlineStr">
+        <is>
+          <t>Компания по переработке отходов: компьютерное зрение на линии сортирует фракции и отбраковывает примеси и загрязнение — выход годного вторсырья растёт, партии чище и дороже при продаже переработчикам.</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n">
@@ -9933,6 +11284,11 @@
           <t>Слуховой центр: почему на бесплатную проверку слуха идут толпы, а аппарат покупает один из десяти, хотя вся маржа именно на нём?</t>
         </is>
       </c>
+      <c r="H271" s="3" t="inlineStr">
+        <is>
+          <t>Слуховой центр: скоринг посетителей по аудиограмме и профилю приоритизирует горячих и подбирает подходящий аппарат, а триггеры возвращают на донастройку — конверсия из бесплатной проверки в покупку растёт.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n">
@@ -9968,6 +11324,11 @@
           <t>Сервис аренды спецтехники: сколько денег съедает экскаватор, что неделю стоит без заказа, пока лизинг, стоянка и зарплата машиниста капают каждый день?</t>
         </is>
       </c>
+      <c r="H272" s="3" t="inlineStr">
+        <is>
+          <t>Сервис аренды спецтехники: на истории заявок, моточасов и простоев ИИ прогнозирует спрос по типам техники и планирует загрузку парка, поднимая утилизацию экскаваторов и сокращая недели простоя между заказами.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n">
@@ -10003,6 +11364,11 @@
           <t>Школа публичных выступлений: куда утекает выручка, когда зал на бесплатном вебинаре полный, а до платного курса доходит меньше трети?</t>
         </is>
       </c>
+      <c r="H273" s="3" t="inlineStr">
+        <is>
+          <t>Школа публичных выступлений: ИИ анализирует записи выступлений — темп, слова-паразиты, паузы, зрительный контакт — и выдаёт мгновенную измеримую обратную связь, ускоряя видимый прогресс ученика и повышая конверсию из вебинара в платный курс.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n">
@@ -10030,12 +11396,17 @@
       </c>
       <c r="F274" s="3" t="inlineStr">
         <is>
-          <t>Закупаем сырьё, проводим шоковую заморозку, фасуем и маркируем, храним при минус восемнадцать, развозим рефрижераторами по сетям и списываем просрочку.</t>
+          <t>Закупаем сырьё, готовим и формуем полуфабрикаты, проводим шоковую заморозку, фасуем и маркируем, храним при минус восемнадцать, развозим рефрижераторами по сетям и списываем просрочку.</t>
         </is>
       </c>
       <c r="G274" s="3" t="inlineStr">
         <is>
           <t>Производитель замороженных продуктов: сколько прибыли тает вместе с продукцией, пока фура стоит на разгрузке у сети, а морозильник не выключить?</t>
+        </is>
+      </c>
+      <c r="H274" s="3" t="inlineStr">
+        <is>
+          <t>Производитель замороженных продуктов: на истории отгрузок и остатков сетей ИИ прогнозирует спрос по SKU и точкам, снижая списания просрочки и дефицит на полке и точнее планируя объём партий.</t>
         </is>
       </c>
     </row>
@@ -10073,6 +11444,11 @@
           <t>Туристическое агентство: почему на подбор тура уходит три часа переписки, а клиент в итоге бронирует тот же пакет напрямую у оператора?</t>
         </is>
       </c>
+      <c r="H275" s="3" t="inlineStr">
+        <is>
+          <t>Туристическое агентство: ИИ-ассистент в переписке по базе туроператоров за минуты подбирает и сравнивает пакеты под запрос клиента, сокращая три часа ручного подбора и удерживая клиента до брони.</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n">
@@ -10108,6 +11484,11 @@
           <t>Лифтовая сервисная компания: почему абонплата за лифт годами одна, а ночные аварийные выезды и дефицит запчастей незаметно съедают всю прибыль договора?</t>
         </is>
       </c>
+      <c r="H276" s="3" t="inlineStr">
+        <is>
+          <t>Лифтовая сервисная компания: на данных журналов, наработки узлов и датчиков ИИ прогнозирует отказы тросов и приводов, сокращая ночные аварийные выезды и ложные вызовы и планируя замены заранее.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n">
@@ -10143,6 +11524,11 @@
           <t>Продюсерский центр артистов: правда ли, что вкладываешься в десятерых, а окупает вложения один, и весь центр живёт на его роялти?</t>
         </is>
       </c>
+      <c r="H277" s="3" t="inlineStr">
+        <is>
+          <t>Продюсерский центр артистов: по ранним метрикам прослушиваний, сохранений и охвата в соцсетях ИИ скорит новые треки и артистов, приоритизируя вложения в тех, кто с большей вероятностью окупится.</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n">
@@ -10178,6 +11564,11 @@
           <t>Оператор платёжных терминалов: куда утекает прибыль, когда половина терминалов приносит копейки, а аренда, связь и инкассация капают за каждый одинаково?</t>
         </is>
       </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>Оператор платёжных терминалов: на истории оборота точек ИИ прогнозирует накопление наличных и строит маршруты инкассации по необходимости, сокращая лишние выезды и подсвечивая мёртвые точки для переноса.</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n">
@@ -10213,6 +11604,11 @@
           <t>Архивная компания: сколько денег заморожено в коробах, за которые клиент платит годами, но так и не забирает и не разрешает уничтожить?</t>
         </is>
       </c>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>Архивная компания: ИИ распознаёт и индексирует содержимое коробов (OCR), давая платный цифровой поиск и выдачу копий без похода к стеллажу, повышая доход с короба и оборачиваемость мест хранения.</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n">
@@ -10248,6 +11644,11 @@
           <t>Издатель видеоигр: почему в игру вложены годы и миллионы, а судьба всего бюджета решается в первые выходные после релиза?</t>
         </is>
       </c>
+      <c r="H280" s="3" t="inlineStr">
+        <is>
+          <t>Издатель видеоигр: ИИ оптимизирует распределение и ставки рекламного бюджета по каналам и странам на данных вишлистов и открутки, снижая стоимость привлечения игрока и риск слить бюджет до релиза.</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n">
@@ -10255,7 +11656,7 @@
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>Магазин фермерских продуктов</t>
+          <t>Магазин настольных игр</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
@@ -10270,17 +11671,22 @@
       </c>
       <c r="E281" s="3" t="inlineStr">
         <is>
-          <t>Магазин фермерских продуктов: как держать маржу на скоропорте, если наценка выше сетевой, а к вечеру половина полки идёт в списание?</t>
+          <t>Магазин настольных игр: как разогнать оборачиваемость полки и превратить демо-столы и клубные вечера в стабильную выручку?</t>
         </is>
       </c>
       <c r="F281" s="3" t="inlineStr">
         <is>
-          <t>Собираем заказы у фермеров, привозим свежее с утра, выкладываем и взвешиваем, продаём в течение дня, уценяем к закрытию и списываем непроданное.</t>
+          <t>Мы закупаем и выкладываем новинки, ведём демо-столы и учим правилам, проводим клубные вечера и турниры, консультируем по выбору, следим за оборачиваемостью полки и допродаём протекторы и аксессуары.</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>Магазин фермерских продуктов: почему покупатель готов платить за фермерское дороже, но свежесть, ради которой он и пришёл, каждый вечер уезжает в мусор?</t>
+          <t>Магазин настольных игр: что убивает маржу, когда игротеки собирают полный зал, а коробки на полке месяцами не находят покупателя?</t>
+        </is>
+      </c>
+      <c r="H281" s="3" t="inlineStr">
+        <is>
+          <t>Магазин настольных игр: на данных клубных вечеров и покупок ИИ рекомендует каждому игроку игры и аксессуары под его предпочтения, повышая оборачиваемость полки и средний чек допродаж.</t>
         </is>
       </c>
     </row>
@@ -10318,6 +11724,11 @@
           <t>B2B-маркетплейс: что мешает заработать, если первую сделку клиенты проводят через площадку, а все следующие — в обход, напрямую с поставщиком?</t>
         </is>
       </c>
+      <c r="H282" s="3" t="inlineStr">
+        <is>
+          <t>B2B-маркетплейс: ИИ выявляет аномалии в поведении пар покупатель-поставщик (обмен контактами, падение повторных заказов), сигнализируя об уходе сделок мимо площадки и запуская удержание, сохраняя комиссионный оборот.</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n">
@@ -10353,6 +11764,11 @@
           <t>Event-агентство: куда исчезает маржа, когда заказчик видит красивый праздник, а вы всю ночь латаете сорванный тайминг и накладки подрядчиков?</t>
         </is>
       </c>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>Event-агентство: на базе прошлых проектов и прайсов подрядчиков ИИ за часы собирает смету и концепцию под бриф, сокращая время подготовки КП и ошибки в расчётах и ускоряя закрытие сделок.</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n">
@@ -10388,6 +11804,11 @@
           <t>Сервис ремонта велосипедов: правда ли, что весь год кормит один весенний вал заявок, а зимой мастерская работает в минус на одной аренде?</t>
         </is>
       </c>
+      <c r="H284" s="3" t="inlineStr">
+        <is>
+          <t>Сервис ремонта велосипедов: на истории ремонтов ИИ прогнозирует, когда клиенту нужно ТО, и шлёт триггерные напоминания и зимние предложения, сглаживая сезонный провал и загружая мастерскую вне пика.</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n">
@@ -10423,6 +11844,11 @@
           <t>Компания по вывозу отходов: сколько прибыли сжигает мусоровоз, который едет по маршруту с полупустыми контейнерами и возвращается порожняком?</t>
         </is>
       </c>
+      <c r="H285" s="3" t="inlineStr">
+        <is>
+          <t>Компания по вывозу отходов: датчики и камеры с ИИ измеряют реальное заполнение контейнеров, чтобы объезжать только полные точки, сокращая порожние рейсы, пробег и расход солярки на маршруте.</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n">
@@ -10458,6 +11884,11 @@
           <t>Ортопедический салон: почему клиент уходит с копеечными стельками, хотя пришёл с проблемой, которую решает корсет в десять раз дороже?</t>
         </is>
       </c>
+      <c r="H286" s="3" t="inlineStr">
+        <is>
+          <t>Ортопедический салон: ИИ анализирует снимок плантоскопа и походку, наглядно показывая клиенту проблему и обоснованно предлагая корсет или обувь, повышая долю апселла и средний чек, а не только продажу стелек.</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n">
@@ -10485,12 +11916,17 @@
       </c>
       <c r="F287" s="3" t="inlineStr">
         <is>
-          <t>Составляем расписание, продаём билеты, выпускаем автобусы на линию, проходим предрейсовый техосмотр и медконтроль, возим пассажиров и обслуживаем парк.</t>
+          <t>Составляем расписание и маршруты, продаём билеты, проходим предрейсовый техосмотр и медконтроль водителей, выпускаем автобусы на линию, возим пассажиров по рейсам и обслуживаем парк в межсменку.</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
           <t>Автобусная транспортная компания: куда утекает выручка, когда утренний рейс набит битком, а дневной идёт по тому же кругу с тремя пассажирами?</t>
+        </is>
+      </c>
+      <c r="H287" s="3" t="inlineStr">
+        <is>
+          <t>Автобусная транспортная компания: на данных загрузки рейсов ИИ гибко управляет ценой билета — скидки на пустые дневные рейсы, — поднимая заполняемость и выручку на рейс без роста расхода топлива.</t>
         </is>
       </c>
     </row>
@@ -10528,6 +11964,11 @@
           <t>Оператор дата-центра: правда ли, что деньги приносят стойки, а половину счёта незаметно съедают кондиционеры, которые эти же стойки и охлаждают?</t>
         </is>
       </c>
+      <c r="H288" s="3" t="inlineStr">
+        <is>
+          <t>Оператор дата-центра: ИИ прогнозирует тепловую и энергонагрузку по стойкам, оптимизируя охлаждение и размещение нагрузки, снижая PUE и распродавая простаивающую мощность, повышая доходность стойки.</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n">
@@ -10563,6 +12004,11 @@
           <t>Сервис возврата налогов: почему берёшь процент только с успеха, но время тратишь одинаково — и на клиента с возвратом, и на того, кому откажут?</t>
         </is>
       </c>
+      <c r="H289" s="3" t="inlineStr">
+        <is>
+          <t>Сервис возврата налогов: по документам и профилю клиента ИИ пред-скринит право на вычет и вероятность одобрения, отсеивая заведомо отказные кейсы, чтобы специалисты тратили время на возвраты, которые окупятся.</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n">
@@ -10598,6 +12044,11 @@
           <t>Организатор фестивалей: правда ли, что годовая прибыль решается за два дня, и один дождь способен смыть всю смету вместе с продажами билетов?</t>
         </is>
       </c>
+      <c r="H290" s="3" t="inlineStr">
+        <is>
+          <t>Организатор фестивалей: на истории продаж, лайнапе и прогнозе погоды ИИ предсказывает посещаемость и динамику продаж билетов, помогая под реальный спрос планировать закупку бара, мерча и персонала.</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n">
@@ -10633,6 +12084,11 @@
           <t>Компания по обслуживанию зданий: куда уходит прибыль, если платят фиксированную сумму, а прорвавшую ночью трубу устраняешь за свой счёт и без сна?</t>
         </is>
       </c>
+      <c r="H291" s="3" t="inlineStr">
+        <is>
+          <t>Компания по обслуживанию зданий: на данных осмотров и датчиков инженерных систем ИИ прогнозирует поломки труб и оборудования, переводя ночные авралы в плановые работы и стабилизируя маржу фиксированного договора.</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n">
@@ -10668,6 +12124,11 @@
           <t>Производитель косметики: почему в баночке крема себестоимость копеечная, а вся прибыль партии уходит в разработку формулы, тару и сертификаты?</t>
         </is>
       </c>
+      <c r="H292" s="3" t="inlineStr">
+        <is>
+          <t>Производитель косметики: ИИ прогнозирует спрос по SKU и каналам до запуска партии, помогая рассчитать тираж и не заморозить деньги в неликвиде, окупая разработку и сертификацию.</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n">
@@ -10703,6 +12164,11 @@
           <t>Платформа перепродажи вещей: что скрывается за ростом объявлений, если каждая вторая сделка уходит в личную переписку мимо вашей комиссии?</t>
         </is>
       </c>
+      <c r="H293" s="3" t="inlineStr">
+        <is>
+          <t>Платформа перепродажи вещей: ИИ подбирает каждому покупателю релевантные объявления в персональной ленте и мгновенно оценивает цену при выставлении, ускоряя продажи внутри площадки и удерживая сделки от ухода в личку.</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n">
@@ -10730,12 +12196,17 @@
       </c>
       <c r="F294" s="3" t="inlineStr">
         <is>
-          <t>Принимаем заказ на кассе и в приложении, собираем на кухне по стандарту, выдаём за минуты, предлагаем допродажу, списываем несобранное и считаем выручку смены.</t>
+          <t>Принимаем заказ на кассе и в приложении, собираем на кухне по стандарту, выдаём за минуты, предлагаем допродажу, следим за поставками и списываем готовое по истечении срока хранения.</t>
         </is>
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
           <t>Сеть быстрого питания: куда утекает маржа, когда очередь на кассе есть, а половина чеков — это акции, промокоды и бесплатная доставка?</t>
+        </is>
+      </c>
+      <c r="H294" s="3" t="inlineStr">
+        <is>
+          <t>Сеть быстрого питания: в приложении и на кассе ИИ предлагает персональные допродажи и наборы под историю заказов, поднимая средний чек и маржу заказа вместо скидочных промокодов.</t>
         </is>
       </c>
     </row>
@@ -10773,6 +12244,11 @@
           <t>Агентство закупочного аутсорсинга: правда ли, что чем больше сэкономишь клиенту, тем меньше он ценит абонентку и тем быстрее решает закупать сам?</t>
         </is>
       </c>
+      <c r="H295" s="3" t="inlineStr">
+        <is>
+          <t>Агентство закупочного аутсорсинга: ИИ анализирует закупки клиента, находит и сравнивает поставщиков и сбивает цены по рынку, увеличивая доказанную экономию на каждом тендере и обосновывая ценность абонентки.</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n">
@@ -10808,6 +12284,11 @@
           <t>Студия 3D-печати: куда утекает прибыль, если принтер печатает одну деталь полдня, а сорвавшийся к утру слой превращает пластик и смену в мусор?</t>
         </is>
       </c>
+      <c r="H296" s="3" t="inlineStr">
+        <is>
+          <t>Студия 3D-печати: камера с ИИ следит за печатью и распознаёт срыв слоя и дефекты на раннем этапе, останавливая брак до конца задания, сокращая расход пластика и переделки и освобождая принтер.</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n">
@@ -10843,6 +12324,11 @@
           <t>Рекламно-производственная компания: почему заказ на вывеску выглядит выгодным, пока переделка макета и повторный выезд монтажников не съедают всю прибыль?</t>
         </is>
       </c>
+      <c r="H297" s="3" t="inlineStr">
+        <is>
+          <t>Рекламно-производственная компания: ИИ по фото фасада за минуты показывает клиенту фотореалистичную вывеску до производства, сокращая переделки макета и повторные выезды монтажников, ускоряя согласование и защищая маржу.</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n">
@@ -10878,6 +12364,11 @@
           <t>Компания по контрактному производству: правда ли, что вы делаете чужой бренд, а вся прибыль решается тем, простаивает линия между заказами или нет?</t>
         </is>
       </c>
+      <c r="H298" s="3" t="inlineStr">
+        <is>
+          <t>Компания по контрактному производству: по техзаданию ИИ быстро считает себестоимость и готовит КП, помогая быстрее закрывать заказы и заполнять окна простоя линии между партиями, поднимая загрузку оборудования.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n">
@@ -10913,6 +12404,11 @@
           <t>Корпоративный учебный центр: почему заказчик легко платит за корпоратив, но торгуется за тренинг, эффект которого не увидит в отчёте на следующий день?</t>
         </is>
       </c>
+      <c r="H299" s="3" t="inlineStr">
+        <is>
+          <t>Корпоративный учебный центр: ИИ анализирует записи звонков продавцов до и после тренинга, измеряя применение навыков и связь с конверсией, давая заказчику цифровое доказательство окупаемости обучения.</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n">
@@ -10948,6 +12444,11 @@
           <t>Сеть зарядных станций для электромобилей: куда уходит прибыль, если станция стоит миллионы, а полдня простаивает, пока рядом заряжают бесплатно у торгового центра?</t>
         </is>
       </c>
+      <c r="H300" s="3" t="inlineStr">
+        <is>
+          <t>Сеть зарядных станций для электромобилей: ИИ прогнозирует загрузку станции по трафику, потоку электромобилей и соседним точкам, помогая размещать станции там, где они окупятся быстрее.</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="n">
@@ -10981,6 +12482,11 @@
       <c r="G301" s="3" t="inlineStr">
         <is>
           <t>Комиссионный магазин: сколько прибыли съедает витрина, забитая вещами, которые сдали полгода назад, а покупатель проходит мимо них каждый день?</t>
+        </is>
+      </c>
+      <c r="H301" s="3" t="inlineStr">
+        <is>
+          <t>Комиссионный магазин: на сроках приёмки и оборачиваемости ИИ рассчитывает динамическую уценку залежавшихся вещей и подсказывает, что не брать на реализацию, освобождая полку от неликвида и ускоряя продажи.</t>
         </is>
       </c>
     </row>

</xml_diff>